<commit_message>
Make group creation a modal and keep merchant names independent
</commit_message>
<xml_diff>
--- a/import-templates/merchant-import-example.xlsx
+++ b/import-templates/merchant-import-example.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="商戶資料" sheetId="1" r:id="R6bf16953a20344e6"/>
-    <sheet name="參數模板" sheetId="2" r:id="Rd044938a4a844e48"/>
-    <sheet name="產品費率" sheetId="3" r:id="R13016af451864d13"/>
-    <sheet name="產品功能" sheetId="4" r:id="R971dd240f2a84966"/>
-    <sheet name="人員資料" sheetId="5" r:id="R4e7e7f88624a4f1f"/>
-    <sheet name="選項清單" sheetId="6" r:id="R4b26ade91602418b"/>
+    <sheet name="商戶資料" sheetId="1" r:id="Rf04d04ef67984b8b"/>
+    <sheet name="參數模板" sheetId="2" r:id="R9a0681b6a3e64757"/>
+    <sheet name="產品費率" sheetId="3" r:id="R96dd373f20824210"/>
+    <sheet name="產品功能" sheetId="4" r:id="R8cfe34bdb83b48f3"/>
+    <sheet name="人員資料" sheetId="5" r:id="R3f0d727f6d0f4f6b"/>
+    <sheet name="選項清單" sheetId="6" r:id="R2e61246cd6804e61"/>
   </sheets>
 </workbook>
 </file>
@@ -130,7 +130,7 @@
     <tableColumn id="1" name="公司代號"/>
     <tableColumn id="2" name="客戶／集團名稱"/>
     <tableColumn id="3" name="公司關係"/>
-    <tableColumn id="4" name="主公司代號"/>
+    <tableColumn id="4" name="母公司代號"/>
     <tableColumn id="5" name="參數模板"/>
     <tableColumn id="6" name="中文名稱"/>
     <tableColumn id="7" name="英文名稱"/>
@@ -561,7 +561,7 @@
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="6" t="str">
-        <v>每家公司一列。先填公司代號；子公司以「主公司代號」連結同一集團的主公司。MCC 可分欄選取。</v>
+        <v>每家公司一列。先填公司代號；子公司以「母公司代號」連結同一集團的母公司。MCC 可分欄選取。</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -624,7 +624,7 @@
         <v>公司關係</v>
       </c>
       <c r="D4" s="10" t="str">
-        <v>主公司代號</v>
+        <v>母公司代號</v>
       </c>
       <c r="E4" s="10" t="str">
         <v>參數模板</v>
@@ -695,14 +695,14 @@
         <v>示例餐飲集團</v>
       </c>
       <c r="C5" s="12" t="str">
-        <v>主公司</v>
+        <v>母公司</v>
       </c>
       <c r="D5" s="12" t="str"/>
       <c r="E5" s="12" t="str">
         <v>餐飲共用參數（示例）</v>
       </c>
       <c r="F5" s="12" t="str">
-        <v>示例餐飲主公司</v>
+        <v>示例餐飲母公司</v>
       </c>
       <c r="G5" s="12" t="str">
         <v>DEMO RESTAURANT HOLDINGS LIMITED</v>
@@ -3376,7 +3376,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R0f697033a10848f8"/>
+    <tablePart r:id="R70020b4aedb04197"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8613,7 +8613,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Rb66c8f74aa834d5c"/>
+    <tablePart r:id="R071faf604ccf4738"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10405,7 +10405,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Racbeec0d60b844ed"/>
+    <tablePart r:id="R77184776b74f4b4b"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11304,7 +11304,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R08ddfdd2c3d34875"/>
+    <tablePart r:id="R8bb00d8d5c7e43a7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12724,7 +12724,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R4ebcfe052e664c3b"/>
+    <tablePart r:id="Ra4993b812c3c468f"/>
   </tableParts>
 </worksheet>
 </file>
@@ -13007,7 +13007,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>主公司</v>
+        <v>母公司</v>
       </c>
       <c r="B3" s="1" t="str">
         <v>5814 · 快餐店</v>

</xml_diff>

<commit_message>
Fix spreadsheet dropdown sources and demonstrate dynamic sample scoring
</commit_message>
<xml_diff>
--- a/import-templates/merchant-import-example.xlsx
+++ b/import-templates/merchant-import-example.xlsx
@@ -2,13 +2,55 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="商戶資料" sheetId="1" r:id="Rf04d04ef67984b8b"/>
-    <sheet name="參數模板" sheetId="2" r:id="R9a0681b6a3e64757"/>
-    <sheet name="產品費率" sheetId="3" r:id="R96dd373f20824210"/>
-    <sheet name="產品功能" sheetId="4" r:id="R8cfe34bdb83b48f3"/>
-    <sheet name="人員資料" sheetId="5" r:id="R3f0d727f6d0f4f6b"/>
-    <sheet name="選項清單" sheetId="6" r:id="R2e61246cd6804e61"/>
+    <sheet name="商戶資料" sheetId="1" r:id="Raa39abbbbe624eb9"/>
+    <sheet name="參數模板" sheetId="2" r:id="Rc0ffffd147294bfc"/>
+    <sheet name="產品費率" sheetId="3" r:id="R8467c63309204c86"/>
+    <sheet name="產品功能" sheetId="4" r:id="Reb8d40dee3534cb8"/>
+    <sheet name="人員資料" sheetId="5" r:id="R6314dad51061481d"/>
+    <sheet name="選項清單" sheetId="6" r:id="Rf85c59b88a0d4874"/>
   </sheets>
+  <definedNames>
+    <definedName name="OATS_Option_1">'選項清單'!$A$2:$A$4</definedName>
+    <definedName name="OATS_Option_2">'選項清單'!$B$2:$B$30</definedName>
+    <definedName name="OATS_Option_3">'選項清單'!$C$2:$C$7</definedName>
+    <definedName name="OATS_Option_4">'選項清單'!$D$2:$D$4</definedName>
+    <definedName name="OATS_Option_5">'選項清單'!$E$2:$E$118</definedName>
+    <definedName name="OATS_Option_6">'選項清單'!$F$2:$F$16</definedName>
+    <definedName name="OATS_Option_7">'選項清單'!$G$2:$G$3</definedName>
+    <definedName name="OATS_Option_8">'選項清單'!$H$2:$H$12</definedName>
+    <definedName name="OATS_Option_9">'選項清單'!$I$2:$I$9</definedName>
+    <definedName name="OATS_Option_10">'選項清單'!$J$2:$J$4</definedName>
+    <definedName name="OATS_Option_11">'選項清單'!$K$2:$K$7</definedName>
+    <definedName name="OATS_Option_12">'選項清單'!$L$2:$L$5</definedName>
+    <definedName name="OATS_Option_13">'選項清單'!$M$2:$M$3</definedName>
+    <definedName name="OATS_Option_14">'選項清單'!$N$2:$N$5</definedName>
+    <definedName name="OATS_Option_15">'選項清單'!$O$2:$O$3</definedName>
+    <definedName name="OATS_Option_16">'選項清單'!$P$2:$P$6</definedName>
+    <definedName name="OATS_Option_17">'選項清單'!$Q$2:$Q$5</definedName>
+    <definedName name="OATS_Option_18">'選項清單'!$R$2:$R$6</definedName>
+    <definedName name="OATS_Option_19">'選項清單'!$S$2:$S$7</definedName>
+    <definedName name="OATS_Option_20">'選項清單'!$T$2:$T$6</definedName>
+    <definedName name="OATS_Option_21">'選項清單'!$U$2:$U$4</definedName>
+    <definedName name="OATS_Option_22">'選項清單'!$V$2:$V$3</definedName>
+    <definedName name="OATS_Option_23">'選項清單'!$W$2:$W$8</definedName>
+    <definedName name="OATS_Option_24">'選項清單'!$X$2:$X$3</definedName>
+    <definedName name="OATS_Option_25">'選項清單'!$Y$2:$Y$3</definedName>
+    <definedName name="OATS_Option_26">'選項清單'!$Z$2:$Z$7</definedName>
+    <definedName name="OATS_Option_27">'選項清單'!$AA$2:$AA$3</definedName>
+    <definedName name="OATS_Option_28">'選項清單'!$AB$2:$AB$4</definedName>
+    <definedName name="OATS_Option_29">'選項清單'!$AC$2:$AC$3</definedName>
+    <definedName name="OATS_Option_30">'選項清單'!$AD$2:$AD$3</definedName>
+    <definedName name="OATS_Option_31">'選項清單'!$AE$2:$AE$3</definedName>
+    <definedName name="OATS_Option_32">'選項清單'!$AF$2:$AF$3</definedName>
+    <definedName name="OATS_Option_33">'選項清單'!$AG$2:$AG$4</definedName>
+    <definedName name="OATS_Option_34">'選項清單'!$AH$2:$AH$30</definedName>
+    <definedName name="OATS_Option_35">'選項清單'!$AI$2:$AI$8</definedName>
+    <definedName name="OATS_Option_36">'選項清單'!$AJ$2:$AJ$7</definedName>
+    <definedName name="OATS_Option_37">'選項清單'!$AK$2:$AK$4</definedName>
+    <definedName name="OATS_Option_38">'選項清單'!$AL$2:$AL$7</definedName>
+    <definedName name="OATS_CompanyIDs">'商戶資料'!$A$5:$A$104</definedName>
+    <definedName name="OATS_TemplateNames">'參數模板'!$A$5:$A$54</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -3344,39 +3386,39 @@
   </sheetData>
   <dataValidations count="10">
     <dataValidation type="list" sqref="C5:C104">
-      <formula1>INDIRECT("'選項清單'!$A$2:$A$4")</formula1>
+      <formula1>OATS_Option_1</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D5:D104">
-      <formula1>INDIRECT("'商戶資料'!$A$5:$A$104")</formula1>
+      <formula1>OATS_CompanyIDs</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E5:E104">
-      <formula1>INDIRECT("'參數模板'!$A$5:$A$54")</formula1>
+      <formula1>OATS_TemplateNames</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I5:I104">
-      <formula1>INDIRECT("'選項清單'!$AH$2:$AH$30")</formula1>
+      <formula1>OATS_Option_34</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="M5:M104">
-      <formula1>INDIRECT("'選項清單'!$AI$2:$AI$8")</formula1>
+      <formula1>OATS_Option_35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="N5:N104">
-      <formula1>INDIRECT("'選項清單'!$W$2:$W$8")</formula1>
+      <formula1>OATS_Option_23</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="O5:O104">
-      <formula1>INDIRECT("'選項清單'!$AJ$2:$AJ$7")</formula1>
+      <formula1>OATS_Option_36</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="U5:U104">
-      <formula1>INDIRECT("'選項清單'!$B$2:$B$30")</formula1>
+      <formula1>OATS_Option_2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="V5:V104">
-      <formula1>INDIRECT("'選項清單'!$B$2:$B$30")</formula1>
+      <formula1>OATS_Option_2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="W5:W104">
-      <formula1>INDIRECT("'選項清單'!$B$2:$B$30")</formula1>
+      <formula1>OATS_Option_2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R70020b4aedb04197"/>
+    <tablePart r:id="R620a7309743b4c5f"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8539,81 +8581,81 @@
   </sheetData>
   <dataValidations count="24">
     <dataValidation type="list" sqref="B5:B54">
-      <formula1>INDIRECT("'選項清單'!$K$2:$K$7")</formula1>
+      <formula1>OATS_Option_11</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C5:C54">
-      <formula1>INDIRECT("'選項清單'!$AH$2:$AH$30")</formula1>
+      <formula1>OATS_Option_34</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D5:D54">
-      <formula1>INDIRECT("'選項清單'!$L$2:$L$5")</formula1>
+      <formula1>OATS_Option_12</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E5:E54">
-      <formula1>INDIRECT("'選項清單'!$N$2:$N$5")</formula1>
+      <formula1>OATS_Option_14</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F5:F54">
-      <formula1>INDIRECT("'選項清單'!$O$2:$O$3")</formula1>
+      <formula1>OATS_Option_15</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="G5:G54">
-      <formula1>INDIRECT("'選項清單'!$P$2:$P$6")</formula1>
+      <formula1>OATS_Option_16</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H5:H54">
-      <formula1>INDIRECT("'選項清單'!$Q$2:$Q$5")</formula1>
+      <formula1>OATS_Option_17</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I5:I54">
-      <formula1>INDIRECT("'選項清單'!$R$2:$R$6")</formula1>
+      <formula1>OATS_Option_18</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="J5:J54">
-      <formula1>INDIRECT("'選項清單'!$S$2:$S$7")</formula1>
+      <formula1>OATS_Option_19</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AA5:AA54">
-      <formula1>INDIRECT("'選項清單'!$V$2:$V$3")</formula1>
+      <formula1>OATS_Option_22</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AC5:AC54">
-      <formula1>INDIRECT("'選項清單'!$AI$2:$AI$8")</formula1>
+      <formula1>OATS_Option_35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AD5:AD54">
-      <formula1>INDIRECT("'選項清單'!$W$2:$W$8")</formula1>
+      <formula1>OATS_Option_23</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AE5:AE54">
-      <formula1>INDIRECT("'選項清單'!$T$2:$T$6")</formula1>
+      <formula1>OATS_Option_20</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AJ5:AJ54">
-      <formula1>INDIRECT("'選項清單'!$AJ$2:$AJ$7")</formula1>
+      <formula1>OATS_Option_36</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AM5:AM54">
-      <formula1>INDIRECT("'選項清單'!$X$2:$X$3")</formula1>
+      <formula1>OATS_Option_24</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AO5:AO54">
-      <formula1>INDIRECT("'選項清單'!$Y$2:$Y$3")</formula1>
+      <formula1>OATS_Option_25</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AP5:AP54">
-      <formula1>INDIRECT("'選項清單'!$AA$2:$AA$3")</formula1>
+      <formula1>OATS_Option_27</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AQ5:AQ54">
-      <formula1>INDIRECT("'選項清單'!$AB$2:$AB$4")</formula1>
+      <formula1>OATS_Option_28</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AR5:AR54">
-      <formula1>INDIRECT("'選項清單'!$AC$2:$AC$3")</formula1>
+      <formula1>OATS_Option_29</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AS5:AS54">
-      <formula1>INDIRECT("'選項清單'!$AD$2:$AD$3")</formula1>
+      <formula1>OATS_Option_30</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AV5:AV54">
-      <formula1>INDIRECT("'選項清單'!$AE$2:$AE$3")</formula1>
+      <formula1>OATS_Option_31</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AW5:AW54">
-      <formula1>INDIRECT("'選項清單'!$AF$2:$AF$3")</formula1>
+      <formula1>OATS_Option_32</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="BK5:BK54">
-      <formula1>INDIRECT("'選項清單'!$AG$2:$AG$4")</formula1>
+      <formula1>OATS_Option_33</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="BR5:BR54">
-      <formula1>INDIRECT("'選項清單'!$M$2:$M$3")</formula1>
+      <formula1>OATS_Option_13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R071faf604ccf4738"/>
+    <tablePart r:id="Ra872517f3890499b"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10376,36 +10418,36 @@
   </sheetData>
   <dataValidations count="9">
     <dataValidation type="list" sqref="A5:A104">
-      <formula1>INDIRECT("'商戶資料'!$A$5:$A$104")</formula1>
+      <formula1>OATS_CompanyIDs</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="B5:B104">
-      <formula1>INDIRECT("'參數模板'!$A$5:$A$54")</formula1>
+      <formula1>OATS_TemplateNames</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C5:C104">
-      <formula1>INDIRECT("'選項清單'!$E$2:$E$118")</formula1>
+      <formula1>OATS_Option_5</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D5:D104">
-      <formula1>INDIRECT("'選項清單'!$G$2:$G$3")</formula1>
+      <formula1>OATS_Option_7</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E5:E104">
-      <formula1>INDIRECT("'選項清單'!$G$2:$G$3")</formula1>
+      <formula1>OATS_Option_7</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F5:F104">
-      <formula1>INDIRECT("'選項清單'!$D$2:$D$4")</formula1>
+      <formula1>OATS_Option_4</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="G5:G104">
-      <formula1>INDIRECT("'選項清單'!$F$2:$F$16")</formula1>
+      <formula1>OATS_Option_6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="M5:M104">
-      <formula1>INDIRECT("'選項清單'!$G$2:$G$3")</formula1>
+      <formula1>OATS_Option_7</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="N5:N104">
-      <formula1>INDIRECT("'選項清單'!$G$2:$G$3")</formula1>
+      <formula1>OATS_Option_7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R77184776b74f4b4b"/>
+    <tablePart r:id="R11e60e7493914aec"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11284,27 +11326,27 @@
   </sheetData>
   <dataValidations count="6">
     <dataValidation type="list" sqref="A5:A104">
-      <formula1>INDIRECT("'商戶資料'!$A$5:$A$104")</formula1>
+      <formula1>OATS_CompanyIDs</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="B5:B104">
-      <formula1>INDIRECT("'參數模板'!$A$5:$A$54")</formula1>
+      <formula1>OATS_TemplateNames</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C5:C104">
-      <formula1>INDIRECT("'選項清單'!$H$2:$H$12")</formula1>
+      <formula1>OATS_Option_8</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D5:D104">
-      <formula1>INDIRECT("'選項清單'!$I$2:$I$9")</formula1>
+      <formula1>OATS_Option_9</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E5:E104">
-      <formula1>INDIRECT("'選項清單'!$G$2:$G$3")</formula1>
+      <formula1>OATS_Option_7</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F5:F104">
-      <formula1>INDIRECT("'選項清單'!$J$2:$J$4")</formula1>
+      <formula1>OATS_Option_10</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R8bb00d8d5c7e43a7"/>
+    <tablePart r:id="Rf6376086eb30407f"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12710,21 +12752,21 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation type="list" sqref="C5:C104">
-      <formula1>INDIRECT("'選項清單'!$AK$2:$AK$4")</formula1>
+      <formula1>OATS_Option_37</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H5:H104">
-      <formula1>INDIRECT("'選項清單'!$AL$2:$AL$7")</formula1>
+      <formula1>OATS_Option_38</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="A5:A104">
-      <formula1>INDIRECT("'商戶資料'!$A$5:$A$104")</formula1>
+      <formula1>OATS_CompanyIDs</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="B5:B104">
-      <formula1>INDIRECT("'參數模板'!$A$5:$A$54")</formula1>
+      <formula1>OATS_TemplateNames</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Ra4993b812c3c468f"/>
+    <tablePart r:id="Re56fc779fc9b4b94"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Apply client review: complete merchant copies, base rates, downline accounts and document downloads
</commit_message>
<xml_diff>
--- a/import-templates/merchant-import-example.xlsx
+++ b/import-templates/merchant-import-example.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet name="商戶資料" sheetId="1" r:id="Raa39abbbbe624eb9"/>
-    <sheet name="參數模板" sheetId="2" r:id="Rc0ffffd147294bfc"/>
-    <sheet name="產品費率" sheetId="3" r:id="R8467c63309204c86"/>
-    <sheet name="產品功能" sheetId="4" r:id="Reb8d40dee3534cb8"/>
-    <sheet name="人員資料" sheetId="5" r:id="R6314dad51061481d"/>
-    <sheet name="選項清單" sheetId="6" r:id="Rf85c59b88a0d4874"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商戶資料" sheetId="1" r:id="Rd8eb093a3a0c45a5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="參數模板" sheetId="2" r:id="R7650a73a969a4e67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="產品費率" sheetId="3" r:id="Rbf4c2c54fc574e5d"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="產品功能" sheetId="4" r:id="Rc44a59fa27304a0a"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人員資料" sheetId="5" r:id="R17beed57f6634248"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="選項清單" sheetId="6" r:id="R643f2ab89041475c"/>
   </sheets>
   <definedNames>
     <definedName name="OATS_Option_1">'選項清單'!$A$2:$A$4</definedName>
     <definedName name="OATS_Option_2">'選項清單'!$B$2:$B$30</definedName>
-    <definedName name="OATS_Option_3">'選項清單'!$C$2:$C$7</definedName>
+    <definedName name="OATS_Option_3">'選項清單'!$C$2:$C$153</definedName>
     <definedName name="OATS_Option_4">'選項清單'!$D$2:$D$4</definedName>
     <definedName name="OATS_Option_5">'選項清單'!$E$2:$E$118</definedName>
     <definedName name="OATS_Option_6">'選項清單'!$F$2:$F$16</definedName>
@@ -45,7 +45,7 @@
     <definedName name="OATS_Option_33">'選項清單'!$AG$2:$AG$4</definedName>
     <definedName name="OATS_Option_34">'選項清單'!$AH$2:$AH$30</definedName>
     <definedName name="OATS_Option_35">'選項清單'!$AI$2:$AI$8</definedName>
-    <definedName name="OATS_Option_36">'選項清單'!$AJ$2:$AJ$7</definedName>
+    <definedName name="OATS_Option_36">'選項清單'!$AJ$2:$AJ$153</definedName>
     <definedName name="OATS_Option_37">'選項清單'!$AK$2:$AK$4</definedName>
     <definedName name="OATS_Option_38">'選項清單'!$AL$2:$AL$7</definedName>
     <definedName name="OATS_CompanyIDs">'商戶資料'!$A$5:$A$104</definedName>
@@ -60,11 +60,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="200" formatCode="@"/>
     <numFmt numFmtId="201" formatCode="0.00"/>
+    <numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -88,6 +89,11 @@
     <font>
       <sz val="10"/>
       <color rgb="FF65728A"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF9C5B00"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -121,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -159,6 +165,12 @@
     <xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="202" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -169,26 +181,26 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Import0" displayName="Import0" ref="A4:X14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="24">
-    <tableColumn id="1" name="公司代號"/>
+    <tableColumn id="1" name="公司代號 *"/>
     <tableColumn id="2" name="客戶／集團名稱"/>
     <tableColumn id="3" name="公司關係"/>
     <tableColumn id="4" name="母公司代號"/>
     <tableColumn id="5" name="參數模板"/>
-    <tableColumn id="6" name="中文名稱"/>
-    <tableColumn id="7" name="英文名稱"/>
-    <tableColumn id="8" name="註冊證書號碼"/>
-    <tableColumn id="9" name="MCC 行業代碼"/>
-    <tableColumn id="10" name="客戶聯絡人"/>
-    <tableColumn id="11" name="聯絡電話"/>
-    <tableColumn id="12" name="聯絡電郵"/>
+    <tableColumn id="6" name="中文名稱 *"/>
+    <tableColumn id="7" name="英文名稱 *"/>
+    <tableColumn id="8" name="註冊證書號碼 *"/>
+    <tableColumn id="9" name="MCC 行業代碼 *"/>
+    <tableColumn id="10" name="客戶聯絡人 *"/>
+    <tableColumn id="11" name="聯絡電話 *"/>
+    <tableColumn id="12" name="聯絡電郵 *"/>
     <tableColumn id="13" name="結算週期"/>
-    <tableColumn id="14" name="幣別"/>
-    <tableColumn id="15" name="開戶銀行"/>
-    <tableColumn id="16" name="開戶銀行行號"/>
-    <tableColumn id="17" name="帳戶名稱"/>
-    <tableColumn id="18" name="銀行帳號"/>
-    <tableColumn id="19" name="業務地址（中文）"/>
-    <tableColumn id="20" name="業務地址（英文）"/>
+    <tableColumn id="14" name="幣別 *"/>
+    <tableColumn id="15" name="開戶銀行 *"/>
+    <tableColumn id="16" name="開戶銀行行號 *"/>
+    <tableColumn id="17" name="帳戶名稱 *"/>
+    <tableColumn id="18" name="銀行帳號 *"/>
+    <tableColumn id="19" name="業務地址（中文） *"/>
+    <tableColumn id="20" name="業務地址（英文） *"/>
     <tableColumn id="21" name="其他 MCC 1"/>
     <tableColumn id="22" name="其他 MCC 2"/>
     <tableColumn id="23" name="其他 MCC 3"/>
@@ -201,8 +213,8 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Import1" displayName="Import1" ref="A4:CJ14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="88">
-    <tableColumn id="1" name="模板名稱"/>
-    <tableColumn id="2" name="套用範圍"/>
+    <tableColumn id="1" name="模板名稱 *"/>
+    <tableColumn id="2" name="套用範圍 *"/>
     <tableColumn id="3" name="MCC 行業代碼"/>
     <tableColumn id="4" name="法律地位"/>
     <tableColumn id="5" name="註冊證書類型"/>
@@ -299,11 +311,11 @@
   <tableColumns count="14">
     <tableColumn id="1" name="公司代號"/>
     <tableColumn id="2" name="模板名稱"/>
-    <tableColumn id="3" name="產品項目"/>
+    <tableColumn id="3" name="產品項目 *"/>
     <tableColumn id="4" name="開通類別"/>
     <tableColumn id="5" name="開通項目"/>
-    <tableColumn id="6" name="收費類型"/>
-    <tableColumn id="7" name="適用範圍"/>
+    <tableColumn id="6" name="收費類型 *"/>
+    <tableColumn id="7" name="適用範圍 *"/>
     <tableColumn id="8" name="費率（%）"/>
     <tableColumn id="9" name="每筆費用（HKD）"/>
     <tableColumn id="10" name="保底（HKD）"/>
@@ -321,9 +333,9 @@
   <tableColumns count="6">
     <tableColumn id="1" name="公司代號"/>
     <tableColumn id="2" name="模板名稱"/>
-    <tableColumn id="3" name="產品類別"/>
-    <tableColumn id="4" name="功能項目"/>
-    <tableColumn id="5" name="開通"/>
+    <tableColumn id="3" name="產品類別 *"/>
+    <tableColumn id="4" name="功能項目 *"/>
+    <tableColumn id="5" name="開通 *"/>
     <tableColumn id="6" name="特計類型"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -335,14 +347,14 @@
   <tableColumns count="11">
     <tableColumn id="1" name="公司代號"/>
     <tableColumn id="2" name="模板名稱"/>
-    <tableColumn id="3" name="人員類型"/>
-    <tableColumn id="4" name="序號"/>
-    <tableColumn id="5" name="姓名"/>
-    <tableColumn id="6" name="英文名"/>
-    <tableColumn id="7" name="英文姓"/>
-    <tableColumn id="8" name="證件類型"/>
-    <tableColumn id="9" name="證件號碼"/>
-    <tableColumn id="10" name="證件有效期"/>
+    <tableColumn id="3" name="人員類型 *"/>
+    <tableColumn id="4" name="序號 *"/>
+    <tableColumn id="5" name="姓名 *"/>
+    <tableColumn id="6" name="英文名 *"/>
+    <tableColumn id="7" name="英文姓 *"/>
+    <tableColumn id="8" name="證件類型 *"/>
+    <tableColumn id="9" name="證件號碼 *"/>
+    <tableColumn id="10" name="證件有效期 *"/>
     <tableColumn id="11" name="出生日期"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -350,198 +362,198 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<theme xmlns="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
-  <themeElements>
-    <clrScheme name="ChatGPT">
-      <dk1>
-        <sysClr val="windowText" lastClr="000000"/>
-      </dk1>
-      <lt1>
-        <sysClr val="window" lastClr="FFFFFF"/>
-      </lt1>
-      <dk2>
-        <srgbClr val="0E2841"/>
-      </dk2>
-      <lt2>
-        <srgbClr val="E8E8E8"/>
-      </lt2>
-      <accent1>
-        <srgbClr val="156082"/>
-      </accent1>
-      <accent2>
-        <srgbClr val="E97132"/>
-      </accent2>
-      <accent3>
-        <srgbClr val="196B24"/>
-      </accent3>
-      <accent4>
-        <srgbClr val="0F9ED5"/>
-      </accent4>
-      <accent5>
-        <srgbClr val="A02B93"/>
-      </accent5>
-      <accent6>
-        <srgbClr val="4EA72E"/>
-      </accent6>
-      <hlink>
-        <srgbClr val="467886"/>
-      </hlink>
-      <folHlink>
-        <srgbClr val="96607D"/>
-      </folHlink>
-    </clrScheme>
-    <fontScheme name="Office">
-      <majorFont>
-        <latin typeface="Calibri Light"/>
-        <ea typeface="Calibri Light"/>
-        <cs typeface="Calibri Light"/>
-      </majorFont>
-      <minorFont>
-        <latin typeface="Calibri"/>
-        <ea typeface="Calibri"/>
-        <cs typeface="Calibri"/>
-      </minorFont>
-    </fontScheme>
-    <fmtScheme name="ChatGPT">
-      <fillStyleLst>
-        <solidFill>
-          <schemeClr val="phClr"/>
-        </solidFill>
-        <gradFill>
-          <gsLst>
-            <gs pos="0">
-              <schemeClr val="phClr">
-                <tint val="67000"/>
-                <lumMod val="110000"/>
-                <satMod val="105000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="50000">
-              <schemeClr val="phClr">
-                <tint val="73000"/>
-                <lumMod val="105000"/>
-                <satMod val="103000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="100000">
-              <schemeClr val="phClr">
-                <tint val="81000"/>
-                <lumMod val="105000"/>
-                <satMod val="109000"/>
-              </schemeClr>
-            </gs>
-          </gsLst>
-          <lin ang="5400000" scaled="0"/>
-        </gradFill>
-        <gradFill>
-          <gsLst>
-            <gs pos="0">
-              <schemeClr val="phClr">
-                <tint val="94000"/>
-                <lumMod val="102000"/>
-                <satMod val="103000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="50000">
-              <schemeClr val="phClr">
-                <shade val="100000"/>
-                <lumMod val="100000"/>
-                <satMod val="110000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="100000">
-              <schemeClr val="phClr">
-                <shade val="78000"/>
-                <lumMod val="99000"/>
-                <satMod val="120000"/>
-              </schemeClr>
-            </gs>
-          </gsLst>
-          <lin ang="5400000" scaled="0"/>
-        </gradFill>
-      </fillStyleLst>
-      <lnStyleLst>
-        <ln w="12700">
-          <solidFill>
-            <schemeClr val="phClr"/>
-          </solidFill>
-          <prstDash val="solid"/>
-        </ln>
-        <ln w="19050">
-          <solidFill>
-            <schemeClr val="phClr"/>
-          </solidFill>
-          <prstDash val="solid"/>
-        </ln>
-        <ln w="25400">
-          <solidFill>
-            <schemeClr val="phClr"/>
-          </solidFill>
-          <prstDash val="solid"/>
-        </ln>
-      </lnStyleLst>
-      <effectStyleLst>
-        <effectStyle>
-          <effectLst/>
-        </effectStyle>
-        <effectStyle>
-          <effectLst/>
-        </effectStyle>
-        <effectStyle>
-          <effectLst>
-            <outerShdw blurRad="57150" dist="19050" dir="5400000">
-              <srgbClr val="000000">
-                <alpha val="63000"/>
-              </srgbClr>
-            </outerShdw>
-          </effectLst>
-        </effectStyle>
-      </effectStyleLst>
-      <bgFillStyleLst>
-        <solidFill>
-          <schemeClr val="phClr"/>
-        </solidFill>
-        <solidFill>
-          <schemeClr val="phClr">
-            <tint val="95000"/>
-            <satMod val="170000"/>
-          </schemeClr>
-        </solidFill>
-        <gradFill>
-          <gsLst>
-            <gs pos="0">
-              <schemeClr val="phClr">
-                <tint val="93000"/>
-                <shade val="98000"/>
-                <lumMod val="102000"/>
-                <satMod val="150000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="50000">
-              <schemeClr val="phClr">
-                <tint val="98000"/>
-                <shade val="90000"/>
-                <lumMod val="103000"/>
-                <satMod val="130000"/>
-              </schemeClr>
-            </gs>
-            <gs pos="100000">
-              <schemeClr val="phClr">
-                <shade val="63000"/>
-                <satMod val="120000"/>
-              </schemeClr>
-            </gs>
-          </gsLst>
-          <lin ang="5400000" scaled="0"/>
-        </gradFill>
-      </bgFillStyleLst>
-    </fmtScheme>
-  </themeElements>
-</theme>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+  <a:themeElements>
+    <a:clrScheme name="ChatGPT">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="ChatGPT">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF168FC7"/>
   </sheetPr>
@@ -629,8 +641,10 @@
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="15" t="str">
+        <v>* 為提交前必填；未完成亦可匯入草稿。產品／人員須填公司代號或模板名稱（二擇一）；子公司須填母公司代號。</v>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -657,7 +671,7 @@
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="10" t="str">
-        <v>公司代號</v>
+        <v>公司代號 *</v>
       </c>
       <c r="B4" s="10" t="str">
         <v>客戶／集團名稱</v>
@@ -672,49 +686,49 @@
         <v>參數模板</v>
       </c>
       <c r="F4" s="10" t="str">
-        <v>中文名稱</v>
+        <v>中文名稱 *</v>
       </c>
       <c r="G4" s="10" t="str">
-        <v>英文名稱</v>
+        <v>英文名稱 *</v>
       </c>
       <c r="H4" s="10" t="str">
-        <v>註冊證書號碼</v>
+        <v>註冊證書號碼 *</v>
       </c>
       <c r="I4" s="10" t="str">
-        <v>MCC 行業代碼</v>
+        <v>MCC 行業代碼 *</v>
       </c>
       <c r="J4" s="10" t="str">
-        <v>客戶聯絡人</v>
+        <v>客戶聯絡人 *</v>
       </c>
       <c r="K4" s="10" t="str">
-        <v>聯絡電話</v>
+        <v>聯絡電話 *</v>
       </c>
       <c r="L4" s="10" t="str">
-        <v>聯絡電郵</v>
+        <v>聯絡電郵 *</v>
       </c>
       <c r="M4" s="10" t="str">
         <v>結算週期</v>
       </c>
       <c r="N4" s="10" t="str">
-        <v>幣別</v>
+        <v>幣別 *</v>
       </c>
       <c r="O4" s="10" t="str">
-        <v>開戶銀行</v>
+        <v>開戶銀行 *</v>
       </c>
       <c r="P4" s="10" t="str">
-        <v>開戶銀行行號</v>
+        <v>開戶銀行行號 *</v>
       </c>
       <c r="Q4" s="10" t="str">
-        <v>帳戶名稱</v>
+        <v>帳戶名稱 *</v>
       </c>
       <c r="R4" s="10" t="str">
-        <v>銀行帳號</v>
+        <v>銀行帳號 *</v>
       </c>
       <c r="S4" s="10" t="str">
-        <v>業務地址（中文）</v>
+        <v>業務地址（中文） *</v>
       </c>
       <c r="T4" s="10" t="str">
-        <v>業務地址（英文）</v>
+        <v>業務地址（英文） *</v>
       </c>
       <c r="U4" s="10" t="str">
         <v>其他 MCC 1</v>
@@ -755,17 +769,39 @@
       <c r="I5" s="12" t="str">
         <v>5812</v>
       </c>
-      <c r="J5" s="12" t="str"/>
-      <c r="K5" s="12" t="str"/>
-      <c r="L5" s="12" t="str"/>
-      <c r="M5" s="12" t="str"/>
-      <c r="N5" s="12" t="str"/>
-      <c r="O5" s="12" t="str"/>
-      <c r="P5" s="12" t="str"/>
-      <c r="Q5" s="12" t="str"/>
-      <c r="R5" s="12" t="str"/>
-      <c r="S5" s="12" t="str"/>
-      <c r="T5" s="12" t="str"/>
+      <c r="J5" s="12" t="str">
+        <v>示例聯絡人 1</v>
+      </c>
+      <c r="K5" s="12" t="str">
+        <v>+85260000001</v>
+      </c>
+      <c r="L5" s="12" t="str">
+        <v>demo1@example.com</v>
+      </c>
+      <c r="M5" s="12" t="str">
+        <v>T2</v>
+      </c>
+      <c r="N5" s="12" t="str">
+        <v>HKD 港元</v>
+      </c>
+      <c r="O5" s="12" t="str">
+        <v>香港上海匯豐銀行有限公司</v>
+      </c>
+      <c r="P5" s="12" t="str">
+        <v>004</v>
+      </c>
+      <c r="Q5" s="12" t="str">
+        <v>DEMO RESTAURANT HOLDINGS LIMITED</v>
+      </c>
+      <c r="R5" s="12" t="str">
+        <v>004000000001</v>
+      </c>
+      <c r="S5" s="12" t="str">
+        <v>香港示例道 1 號</v>
+      </c>
+      <c r="T5" s="12" t="str">
+        <v>1 DEMO ROAD, HONG KONG</v>
+      </c>
       <c r="U5" s="12" t="str">
         <v>5814</v>
       </c>
@@ -801,17 +837,39 @@
       <c r="I6" s="12" t="str">
         <v>5812</v>
       </c>
-      <c r="J6" s="12" t="str"/>
-      <c r="K6" s="12" t="str"/>
-      <c r="L6" s="12" t="str"/>
-      <c r="M6" s="12" t="str"/>
-      <c r="N6" s="12" t="str"/>
-      <c r="O6" s="12" t="str"/>
-      <c r="P6" s="12" t="str"/>
-      <c r="Q6" s="12" t="str"/>
-      <c r="R6" s="12" t="str"/>
-      <c r="S6" s="12" t="str"/>
-      <c r="T6" s="12" t="str"/>
+      <c r="J6" s="12" t="str">
+        <v>示例聯絡人 2</v>
+      </c>
+      <c r="K6" s="12" t="str">
+        <v>+85260000002</v>
+      </c>
+      <c r="L6" s="12" t="str">
+        <v>demo2@example.com</v>
+      </c>
+      <c r="M6" s="12" t="str">
+        <v>T2</v>
+      </c>
+      <c r="N6" s="12" t="str">
+        <v>HKD 港元</v>
+      </c>
+      <c r="O6" s="12" t="str">
+        <v>香港上海匯豐銀行有限公司</v>
+      </c>
+      <c r="P6" s="12" t="str">
+        <v>004</v>
+      </c>
+      <c r="Q6" s="12" t="str">
+        <v>DEMO RESTAURANT A LIMITED</v>
+      </c>
+      <c r="R6" s="12" t="str">
+        <v>004000000002</v>
+      </c>
+      <c r="S6" s="12" t="str">
+        <v>香港示例道 1 號</v>
+      </c>
+      <c r="T6" s="12" t="str">
+        <v>1 DEMO ROAD, HONG KONG</v>
+      </c>
       <c r="U6" s="12" t="str"/>
       <c r="V6" s="12" t="str"/>
       <c r="W6" s="12" t="str"/>
@@ -845,17 +903,39 @@
       <c r="I7" s="12" t="str">
         <v>5814</v>
       </c>
-      <c r="J7" s="12" t="str"/>
-      <c r="K7" s="12" t="str"/>
-      <c r="L7" s="12" t="str"/>
-      <c r="M7" s="12" t="str"/>
-      <c r="N7" s="12" t="str"/>
-      <c r="O7" s="12" t="str"/>
-      <c r="P7" s="12" t="str"/>
-      <c r="Q7" s="12" t="str"/>
-      <c r="R7" s="12" t="str"/>
-      <c r="S7" s="12" t="str"/>
-      <c r="T7" s="12" t="str"/>
+      <c r="J7" s="12" t="str">
+        <v>示例聯絡人 3</v>
+      </c>
+      <c r="K7" s="12" t="str">
+        <v>+85260000003</v>
+      </c>
+      <c r="L7" s="12" t="str">
+        <v>demo3@example.com</v>
+      </c>
+      <c r="M7" s="12" t="str">
+        <v>T2</v>
+      </c>
+      <c r="N7" s="12" t="str">
+        <v>HKD 港元</v>
+      </c>
+      <c r="O7" s="12" t="str">
+        <v>香港上海匯豐銀行有限公司</v>
+      </c>
+      <c r="P7" s="12" t="str">
+        <v>004</v>
+      </c>
+      <c r="Q7" s="12" t="str">
+        <v>DEMO RESTAURANT B LIMITED</v>
+      </c>
+      <c r="R7" s="12" t="str">
+        <v>004000000003</v>
+      </c>
+      <c r="S7" s="12" t="str">
+        <v>香港示例道 1 號</v>
+      </c>
+      <c r="T7" s="12" t="str">
+        <v>1 DEMO ROAD, HONG KONG</v>
+      </c>
       <c r="U7" s="12" t="str"/>
       <c r="V7" s="12" t="str"/>
       <c r="W7" s="12" t="str"/>
@@ -3418,13 +3498,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R620a7309743b4c5f"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77dba84da96f491e"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF168FC7"/>
   </sheetPr>
@@ -3704,8 +3784,10 @@
       <c r="CI2" s="4"/>
       <c r="CJ2" s="4"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="15" t="str">
+        <v>* 為提交前必填；未完成亦可匯入草稿。產品／人員須填公司代號或模板名稱（二擇一）；子公司須填母公司代號。</v>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -3796,10 +3878,10 @@
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="10" t="str">
-        <v>模板名稱</v>
+        <v>模板名稱 *</v>
       </c>
       <c r="B4" s="10" t="str">
-        <v>套用範圍</v>
+        <v>套用範圍 *</v>
       </c>
       <c r="C4" s="10" t="str">
         <v>MCC 行業代碼</v>
@@ -8655,13 +8737,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Ra872517f3890499b"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc00a07d1d9a34b26"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF168FC7"/>
   </sheetPr>
@@ -8719,8 +8801,10 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="15" t="str">
+        <v>* 為提交前必填；未完成亦可匯入草稿。產品／人員須填公司代號或模板名稱（二擇一）；子公司須填母公司代號。</v>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -8743,7 +8827,7 @@
         <v>模板名稱</v>
       </c>
       <c r="C4" s="10" t="str">
-        <v>產品項目</v>
+        <v>產品項目 *</v>
       </c>
       <c r="D4" s="10" t="str">
         <v>開通類別</v>
@@ -8752,10 +8836,10 @@
         <v>開通項目</v>
       </c>
       <c r="F4" s="10" t="str">
-        <v>收費類型</v>
+        <v>收費類型 *</v>
       </c>
       <c r="G4" s="10" t="str">
-        <v>適用範圍</v>
+        <v>適用範圍 *</v>
       </c>
       <c r="H4" s="10" t="str">
         <v>費率（%）</v>
@@ -10447,13 +10531,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R11e60e7493914aec"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d6d32d28d94b38"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF168FC7"/>
   </sheetPr>
@@ -10487,8 +10571,10 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="15" t="str">
+        <v>* 為提交前必填；未完成亦可匯入草稿。產品／人員須填公司代號或模板名稱（二擇一）；子公司須填母公司代號。</v>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -10503,13 +10589,13 @@
         <v>模板名稱</v>
       </c>
       <c r="C4" s="10" t="str">
-        <v>產品類別</v>
+        <v>產品類別 *</v>
       </c>
       <c r="D4" s="10" t="str">
-        <v>功能項目</v>
+        <v>功能項目 *</v>
       </c>
       <c r="E4" s="10" t="str">
-        <v>開通</v>
+        <v>開通 *</v>
       </c>
       <c r="F4" s="10" t="str">
         <v>特計類型</v>
@@ -11346,13 +11432,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Rf6376086eb30407f"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91da6336a3b64eaa"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF168FC7"/>
   </sheetPr>
@@ -11401,8 +11487,10 @@
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="15" t="str">
+        <v>* 為提交前必填；未完成亦可匯入草稿。產品／人員須填公司代號或模板名稱（二擇一）；子公司須填母公司代號。</v>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -11422,71 +11510,131 @@
         <v>模板名稱</v>
       </c>
       <c r="C4" s="10" t="str">
-        <v>人員類型</v>
+        <v>人員類型 *</v>
       </c>
       <c r="D4" s="10" t="str">
-        <v>序號</v>
+        <v>序號 *</v>
       </c>
       <c r="E4" s="10" t="str">
-        <v>姓名</v>
+        <v>姓名 *</v>
       </c>
       <c r="F4" s="10" t="str">
-        <v>英文名</v>
+        <v>英文名 *</v>
       </c>
       <c r="G4" s="10" t="str">
-        <v>英文姓</v>
+        <v>英文姓 *</v>
       </c>
       <c r="H4" s="10" t="str">
-        <v>證件類型</v>
+        <v>證件類型 *</v>
       </c>
       <c r="I4" s="10" t="str">
-        <v>證件號碼</v>
+        <v>證件號碼 *</v>
       </c>
       <c r="J4" s="10" t="str">
-        <v>證件有效期</v>
+        <v>證件有效期 *</v>
       </c>
       <c r="K4" s="10" t="str">
         <v>出生日期</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
+      <c r="A5" s="12" t="str">
+        <v>MAIN</v>
+      </c>
+      <c r="B5" s="12" t="str"/>
+      <c r="C5" s="12" t="str">
+        <v>董事</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <v>示例董事甲</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <v>DEMO</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <v>CHAN</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <v>護照</v>
+      </c>
+      <c r="I5" s="12" t="str">
+        <v>DEMO0001</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>47848</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <v>29221</v>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
+      <c r="A6" s="12" t="str">
+        <v>SUB-A</v>
+      </c>
+      <c r="B6" s="12" t="str"/>
+      <c r="C6" s="12" t="str">
+        <v>董事</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="12" t="str">
+        <v>示例董事乙</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <v>DEMO</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <v>LEE</v>
+      </c>
+      <c r="H6" s="12" t="str">
+        <v>護照</v>
+      </c>
+      <c r="I6" s="12" t="str">
+        <v>DEMO0002</v>
+      </c>
+      <c r="J6" s="16" t="n">
+        <v>47848</v>
+      </c>
+      <c r="K6" s="16" t="n">
+        <v>31048</v>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
+      <c r="A7" s="12" t="str">
+        <v>SUB-B</v>
+      </c>
+      <c r="B7" s="12" t="str"/>
+      <c r="C7" s="12" t="str">
+        <v>董事</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="12" t="str">
+        <v>示例董事丙</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <v>DEMO</v>
+      </c>
+      <c r="G7" s="12" t="str">
+        <v>WONG</v>
+      </c>
+      <c r="H7" s="12" t="str">
+        <v>護照</v>
+      </c>
+      <c r="I7" s="12" t="str">
+        <v>DEMO0003</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>47848</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>32143</v>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="12"/>
@@ -12766,7 +12914,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Re56fc779fc9b4b94"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd04ad15448054da7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12939,7 +13087,7 @@
         <v>5812 · 餐廳</v>
       </c>
       <c r="C2" s="1" t="str">
-        <v>渣打銀行（香港）</v>
+        <v>渣打銀行(香港)有限公司</v>
       </c>
       <c r="D2" s="1" t="str">
         <v>Regional</v>
@@ -13038,7 +13186,7 @@
         <v>T1</v>
       </c>
       <c r="AJ2" s="1" t="str">
-        <v>渣打銀行（香港）</v>
+        <v>渣打銀行(香港)有限公司</v>
       </c>
       <c r="AK2" s="1" t="str">
         <v>董事</v>
@@ -13055,7 +13203,7 @@
         <v>5814 · 快餐店</v>
       </c>
       <c r="C3" s="1" t="str">
-        <v>香港上海滙豐銀行</v>
+        <v>香港上海匯豐銀行有限公司</v>
       </c>
       <c r="D3" s="1" t="str">
         <v>Blended</v>
@@ -13154,7 +13302,7 @@
         <v>T2</v>
       </c>
       <c r="AJ3" s="1" t="str">
-        <v>香港上海滙豐銀行</v>
+        <v>香港上海匯豐銀行有限公司</v>
       </c>
       <c r="AK3" s="1" t="str">
         <v>授權簽名人</v>
@@ -13171,7 +13319,7 @@
         <v>5411 · 超市／雜貨店</v>
       </c>
       <c r="C4" s="1" t="str">
-        <v>中國銀行（香港）</v>
+        <v>CREDIT AGRICOLE CORPORATE AND INVESTMENT BANK</v>
       </c>
       <c r="D4" s="1" t="str">
         <v>Wallet</v>
@@ -13248,7 +13396,7 @@
         <v>T3</v>
       </c>
       <c r="AJ4" s="1" t="str">
-        <v>中國銀行（香港）</v>
+        <v>CREDIT AGRICOLE CORPORATE AND INVESTMENT BANK</v>
       </c>
       <c r="AK4" s="1" t="str">
         <v>股東</v>
@@ -13263,7 +13411,7 @@
         <v>5311 · 百貨公司</v>
       </c>
       <c r="C5" s="1" t="str">
-        <v>東亞銀行</v>
+        <v>花旗銀行</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="str">
@@ -13330,7 +13478,7 @@
         <v>T5</v>
       </c>
       <c r="AJ5" s="1" t="str">
-        <v>東亞銀行</v>
+        <v>花旗銀行</v>
       </c>
       <c r="AK5" s="1"/>
       <c r="AL5" s="1" t="str">
@@ -13343,7 +13491,7 @@
         <v>5651 · 服飾零售</v>
       </c>
       <c r="C6" s="1" t="str">
-        <v>星展銀行（香港）</v>
+        <v>JPMORGAN CHASE BANK, N.A.</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="str">
@@ -13404,7 +13552,7 @@
         <v>T7</v>
       </c>
       <c r="AJ6" s="1" t="str">
-        <v>星展銀行（香港）</v>
+        <v>JPMORGAN CHASE BANK, N.A.</v>
       </c>
       <c r="AK6" s="1"/>
       <c r="AL6" s="1" t="str">
@@ -13417,7 +13565,7 @@
         <v>7230 · 美容美髮</v>
       </c>
       <c r="C7" s="1" t="str">
-        <v>恒生銀行</v>
+        <v>中國建設銀行(亞洲)股份有限公司</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="str">
@@ -13472,7 +13620,7 @@
         <v>D0</v>
       </c>
       <c r="AJ7" s="1" t="str">
-        <v>恒生銀行</v>
+        <v>中國建設銀行(亞洲)股份有限公司</v>
       </c>
       <c r="AK7" s="1"/>
       <c r="AL7" s="1" t="str">
@@ -13484,7 +13632,9 @@
       <c r="B8" s="1" t="str">
         <v>5462 · 麵包糕餅店</v>
       </c>
-      <c r="C8" s="1"/>
+      <c r="C8" s="1" t="str">
+        <v>中國銀行(香港)有限公司</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="str">
         <v>收單／VISA 收單-分期消費</v>
@@ -13531,7 +13681,9 @@
       <c r="AI8" s="1" t="str">
         <v>D1</v>
       </c>
-      <c r="AJ8" s="1"/>
+      <c r="AJ8" s="1" t="str">
+        <v>中國銀行(香港)有限公司</v>
+      </c>
       <c r="AK8" s="1"/>
       <c r="AL8" s="1"/>
     </row>
@@ -13540,7 +13692,9 @@
       <c r="B9" s="1" t="str">
         <v>5945 · 玩具遊戲零售</v>
       </c>
-      <c r="C9" s="1"/>
+      <c r="C9" s="1" t="str">
+        <v>東亞銀行有限公司</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="str">
         <v>收單／八達通-消費</v>
@@ -13583,7 +13737,9 @@
         <v>5945 · 玩具遊戲零售</v>
       </c>
       <c r="AI9" s="1"/>
-      <c r="AJ9" s="1"/>
+      <c r="AJ9" s="1" t="str">
+        <v>東亞銀行有限公司</v>
+      </c>
       <c r="AK9" s="1"/>
       <c r="AL9" s="1"/>
     </row>
@@ -13592,7 +13748,9 @@
       <c r="B10" s="1" t="str">
         <v>5977 · 化妝品店</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="str">
+        <v>星展銀行(香港)有限公司</v>
+      </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="str">
         <v>CTV／VISA 線上消費</v>
@@ -13633,7 +13791,9 @@
         <v>5977 · 化妝品店</v>
       </c>
       <c r="AI10" s="1"/>
-      <c r="AJ10" s="1"/>
+      <c r="AJ10" s="1" t="str">
+        <v>星展銀行(香港)有限公司</v>
+      </c>
       <c r="AK10" s="1"/>
       <c r="AL10" s="1"/>
     </row>
@@ -13642,7 +13802,9 @@
       <c r="B11" s="1" t="str">
         <v>7298 · 健康美容中心</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="str">
+        <v>中信銀行(國際)有限公司</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="str">
         <v>CTV／MASTERCARD 線上消費</v>
@@ -13683,7 +13845,9 @@
         <v>7298 · 健康美容中心</v>
       </c>
       <c r="AI11" s="1"/>
-      <c r="AJ11" s="1"/>
+      <c r="AJ11" s="1" t="str">
+        <v>中信銀行(國際)有限公司</v>
+      </c>
       <c r="AK11" s="1"/>
       <c r="AL11" s="1"/>
     </row>
@@ -13692,7 +13856,9 @@
       <c r="B12" s="1" t="str">
         <v>5944 · 珠寶鐘錶</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="str">
+        <v>招商永隆銀行有限公司</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="str">
         <v>CTV／JCB 線上消費</v>
@@ -13733,7 +13899,9 @@
         <v>5944 · 珠寶鐘錶</v>
       </c>
       <c r="AI12" s="1"/>
-      <c r="AJ12" s="1"/>
+      <c r="AJ12" s="1" t="str">
+        <v>招商永隆銀行有限公司</v>
+      </c>
       <c r="AK12" s="1"/>
       <c r="AL12" s="1"/>
     </row>
@@ -13742,7 +13910,9 @@
       <c r="B13" s="1" t="str">
         <v>4722 · 旅行社</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="str">
+        <v>OVERSEA-CHINESE BANKING CORPORATION LTD.</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="str">
         <v>CTV／UNIONPAY 線上消費</v>
@@ -13781,7 +13951,9 @@
         <v>4722 · 旅行社</v>
       </c>
       <c r="AI13" s="1"/>
-      <c r="AJ13" s="1"/>
+      <c r="AJ13" s="1" t="str">
+        <v>OVERSEA-CHINESE BANKING CORPORATION LTD.</v>
+      </c>
       <c r="AK13" s="1"/>
       <c r="AL13" s="1"/>
     </row>
@@ -13790,7 +13962,9 @@
       <c r="B14" s="1" t="str">
         <v>7011 · 酒店住宿</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="str">
+        <v>恒生銀行有限公司</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="str">
         <v>CNP／VISA 線上消費</v>
@@ -13829,7 +14003,9 @@
         <v>7011 · 酒店住宿</v>
       </c>
       <c r="AI14" s="1"/>
-      <c r="AJ14" s="1"/>
+      <c r="AJ14" s="1" t="str">
+        <v>恒生銀行有限公司</v>
+      </c>
       <c r="AK14" s="1"/>
       <c r="AL14" s="1"/>
     </row>
@@ -13838,7 +14014,9 @@
       <c r="B15" s="1" t="str">
         <v>5722 · 家用電器</v>
       </c>
-      <c r="C15" s="1"/>
+      <c r="C15" s="1" t="str">
+        <v>上海商業銀行有限公司</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="str">
         <v>CNP／MASTERCARD 線上消費</v>
@@ -13877,7 +14055,9 @@
         <v>5722 · 家用電器</v>
       </c>
       <c r="AI15" s="1"/>
-      <c r="AJ15" s="1"/>
+      <c r="AJ15" s="1" t="str">
+        <v>上海商業銀行有限公司</v>
+      </c>
       <c r="AK15" s="1"/>
       <c r="AL15" s="1"/>
     </row>
@@ -13886,7 +14066,9 @@
       <c r="B16" s="1" t="str">
         <v>5732 · 電子產品零售</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1" t="str">
+        <v>交通銀行股份有限公司</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="str">
         <v>CNP／VISA 線上分期消費</v>
@@ -13925,7 +14107,9 @@
         <v>5732 · 電子產品零售</v>
       </c>
       <c r="AI16" s="1"/>
-      <c r="AJ16" s="1"/>
+      <c r="AJ16" s="1" t="str">
+        <v>交通銀行股份有限公司</v>
+      </c>
       <c r="AK16" s="1"/>
       <c r="AL16" s="1"/>
     </row>
@@ -13934,7 +14118,9 @@
       <c r="B17" s="1" t="str">
         <v>7995 · 博彩</v>
       </c>
-      <c r="C17" s="1"/>
+      <c r="C17" s="1" t="str">
+        <v>大眾銀行(香港)有限公司</v>
+      </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="str">
         <v>CNP／DINERSCLUB 線上消費</v>
@@ -13971,7 +14157,9 @@
         <v>7995 · 博彩</v>
       </c>
       <c r="AI17" s="1"/>
-      <c r="AJ17" s="1"/>
+      <c r="AJ17" s="1" t="str">
+        <v>大眾銀行(香港)有限公司</v>
+      </c>
       <c r="AK17" s="1"/>
       <c r="AL17" s="1"/>
     </row>
@@ -13980,7 +14168,9 @@
       <c r="B18" s="1" t="str">
         <v>6010 · 金融機構—人工提現</v>
       </c>
-      <c r="C18" s="1"/>
+      <c r="C18" s="1" t="str">
+        <v>華僑銀行(香港)有限公司</v>
+      </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="str">
         <v>CNP／JCB 線上消費</v>
@@ -14017,7 +14207,9 @@
         <v>6010 · 金融機構—人工提現</v>
       </c>
       <c r="AI18" s="1"/>
-      <c r="AJ18" s="1"/>
+      <c r="AJ18" s="1" t="str">
+        <v>華僑銀行(香港)有限公司</v>
+      </c>
       <c r="AK18" s="1"/>
       <c r="AL18" s="1"/>
     </row>
@@ -14026,7 +14218,9 @@
       <c r="B19" s="1" t="str">
         <v>6011 · 金融機構—自動提現</v>
       </c>
-      <c r="C19" s="1"/>
+      <c r="C19" s="1" t="str">
+        <v>大有銀行有限公司</v>
+      </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="str">
         <v>CNP／AMERICAEXPRESS 線上消費</v>
@@ -14063,7 +14257,9 @@
         <v>6011 · 金融機構—自動提現</v>
       </c>
       <c r="AI19" s="1"/>
-      <c r="AJ19" s="1"/>
+      <c r="AJ19" s="1" t="str">
+        <v>大有銀行有限公司</v>
+      </c>
       <c r="AK19" s="1"/>
       <c r="AL19" s="1"/>
     </row>
@@ -14072,7 +14268,9 @@
       <c r="B20" s="1" t="str">
         <v>6012 · 金融機構—商品服務</v>
       </c>
-      <c r="C20" s="1"/>
+      <c r="C20" s="1" t="str">
+        <v>集友銀行有限公司</v>
+      </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="str">
         <v>CNP／UNIONPAY 線上消費</v>
@@ -14109,7 +14307,9 @@
         <v>6012 · 金融機構—商品服務</v>
       </c>
       <c r="AI20" s="1"/>
-      <c r="AJ20" s="1"/>
+      <c r="AJ20" s="1" t="str">
+        <v>集友銀行有限公司</v>
+      </c>
       <c r="AK20" s="1"/>
       <c r="AL20" s="1"/>
     </row>
@@ -14118,7 +14318,9 @@
       <c r="B21" s="1" t="str">
         <v>6051 · 準現金／外幣兌換</v>
       </c>
-      <c r="C21" s="1"/>
+      <c r="C21" s="1" t="str">
+        <v>大新銀行有限公司</v>
+      </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="str">
         <v>CNP／VISA TOKEN線上消費</v>
@@ -14155,7 +14357,9 @@
         <v>6051 · 準現金／外幣兌換</v>
       </c>
       <c r="AI21" s="1"/>
-      <c r="AJ21" s="1"/>
+      <c r="AJ21" s="1" t="str">
+        <v>大新銀行有限公司</v>
+      </c>
       <c r="AK21" s="1"/>
       <c r="AL21" s="1"/>
     </row>
@@ -14164,7 +14368,9 @@
       <c r="B22" s="1" t="str">
         <v>5122 · 藥品批發</v>
       </c>
-      <c r="C22" s="1"/>
+      <c r="C22" s="1" t="str">
+        <v>創興銀行有限公司</v>
+      </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="str">
         <v>CNP／MASTERCARD TOKEN線上消費</v>
@@ -14201,7 +14407,9 @@
         <v>5122 · 藥品批發</v>
       </c>
       <c r="AI22" s="1"/>
-      <c r="AJ22" s="1"/>
+      <c r="AJ22" s="1" t="str">
+        <v>創興銀行有限公司</v>
+      </c>
       <c r="AK22" s="1"/>
       <c r="AL22" s="1"/>
     </row>
@@ -14210,7 +14418,9 @@
       <c r="B23" s="1" t="str">
         <v>5912 · 藥房</v>
       </c>
-      <c r="C23" s="1"/>
+      <c r="C23" s="1" t="str">
+        <v>南洋商業銀行有限公司</v>
+      </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="str">
         <v>CNP／JCB TOKEN線上消費</v>
@@ -14247,7 +14457,9 @@
         <v>5912 · 藥房</v>
       </c>
       <c r="AI23" s="1"/>
-      <c r="AJ23" s="1"/>
+      <c r="AJ23" s="1" t="str">
+        <v>南洋商業銀行有限公司</v>
+      </c>
       <c r="AK23" s="1"/>
       <c r="AL23" s="1"/>
     </row>
@@ -14256,7 +14468,9 @@
       <c r="B24" s="1" t="str">
         <v>5962 · 電話銷售</v>
       </c>
-      <c r="C24" s="1"/>
+      <c r="C24" s="1" t="str">
+        <v>UCO BANK</v>
+      </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="str">
         <v>CNP／AMERICAEXPRESS TOKEN線上消費</v>
@@ -14293,7 +14507,9 @@
         <v>5962 · 電話銷售</v>
       </c>
       <c r="AI24" s="1"/>
-      <c r="AJ24" s="1"/>
+      <c r="AJ24" s="1" t="str">
+        <v>UCO BANK</v>
+      </c>
       <c r="AK24" s="1"/>
       <c r="AL24" s="1"/>
     </row>
@@ -14302,7 +14518,9 @@
       <c r="B25" s="1" t="str">
         <v>5966 · 外呼銷售</v>
       </c>
-      <c r="C25" s="1"/>
+      <c r="C25" s="1" t="str">
+        <v>KEB HANA BANK</v>
+      </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="str">
         <v>CNP／UNIONPAY TOKEN線上消費</v>
@@ -14339,7 +14557,9 @@
         <v>5966 · 外呼銷售</v>
       </c>
       <c r="AI25" s="1"/>
-      <c r="AJ25" s="1"/>
+      <c r="AJ25" s="1" t="str">
+        <v>KEB HANA BANK</v>
+      </c>
       <c r="AK25" s="1"/>
       <c r="AL25" s="1"/>
     </row>
@@ -14348,7 +14568,9 @@
       <c r="B26" s="1" t="str">
         <v>5967 · 成人內容</v>
       </c>
-      <c r="C26" s="1"/>
+      <c r="C26" s="1" t="str">
+        <v>MUFG BANK, LTD.</v>
+      </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="str">
         <v>CNP／VISA TOKEN預授權</v>
@@ -14385,7 +14607,9 @@
         <v>5967 · 成人內容</v>
       </c>
       <c r="AI26" s="1"/>
-      <c r="AJ26" s="1"/>
+      <c r="AJ26" s="1" t="str">
+        <v>MUFG BANK, LTD.</v>
+      </c>
       <c r="AK26" s="1"/>
       <c r="AL26" s="1"/>
     </row>
@@ -14394,7 +14618,9 @@
       <c r="B27" s="1" t="str">
         <v>4829 · 匯款／轉帳</v>
       </c>
-      <c r="C27" s="1"/>
+      <c r="C27" s="1" t="str">
+        <v>BANGKOK BANK PUBLIC COMPANY LIMITED</v>
+      </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="str">
         <v>CNP／MASTERCARD TOKEN預授權</v>
@@ -14431,7 +14657,9 @@
         <v>4829 · 匯款／轉帳</v>
       </c>
       <c r="AI27" s="1"/>
-      <c r="AJ27" s="1"/>
+      <c r="AJ27" s="1" t="str">
+        <v>BANGKOK BANK PUBLIC COMPANY LIMITED</v>
+      </c>
       <c r="AK27" s="1"/>
       <c r="AL27" s="1"/>
     </row>
@@ -14440,7 +14668,9 @@
       <c r="B28" s="1" t="str">
         <v>5993 · 煙草</v>
       </c>
-      <c r="C28" s="1"/>
+      <c r="C28" s="1" t="str">
+        <v>INDIAN OVERSEAS BANK</v>
+      </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="str">
         <v>CNP／JCB TOKEN預授權</v>
@@ -14477,7 +14707,9 @@
         <v>5993 · 煙草</v>
       </c>
       <c r="AI28" s="1"/>
-      <c r="AJ28" s="1"/>
+      <c r="AJ28" s="1" t="str">
+        <v>INDIAN OVERSEAS BANK</v>
+      </c>
       <c r="AK28" s="1"/>
       <c r="AL28" s="1"/>
     </row>
@@ -14486,7 +14718,9 @@
       <c r="B29" s="1" t="str">
         <v>7273 · 約會交友服務</v>
       </c>
-      <c r="C29" s="1"/>
+      <c r="C29" s="1" t="str">
+        <v>DEUTSCHE BANK AG</v>
+      </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1" t="str">
         <v>CNP／AMERICAEXPRESS TOKEN預授權</v>
@@ -14523,7 +14757,9 @@
         <v>7273 · 約會交友服務</v>
       </c>
       <c r="AI29" s="1"/>
-      <c r="AJ29" s="1"/>
+      <c r="AJ29" s="1" t="str">
+        <v>DEUTSCHE BANK AG</v>
+      </c>
       <c r="AK29" s="1"/>
       <c r="AL29" s="1"/>
     </row>
@@ -14532,7 +14768,9 @@
       <c r="B30" s="1" t="str">
         <v>8062 · 醫院</v>
       </c>
-      <c r="C30" s="1"/>
+      <c r="C30" s="1" t="str">
+        <v>BANK OF AMERICA, NATIONAL ASSOCIATION</v>
+      </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="str">
         <v>CNP／UNIONPAY TOKEN預授權</v>
@@ -14569,14 +14807,18 @@
         <v>8062 · 醫院</v>
       </c>
       <c r="AI30" s="1"/>
-      <c r="AJ30" s="1"/>
+      <c r="AJ30" s="1" t="str">
+        <v>BANK OF AMERICA, NATIONAL ASSOCIATION</v>
+      </c>
       <c r="AK30" s="1"/>
       <c r="AL30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
+      <c r="C31" s="1" t="str">
+        <v>BNP PARIBAS</v>
+      </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1" t="str">
         <v>CNP／VISA 線上預授權</v>
@@ -14611,14 +14853,18 @@
       <c r="AG31" s="1"/>
       <c r="AH31" s="1"/>
       <c r="AI31" s="1"/>
-      <c r="AJ31" s="1"/>
+      <c r="AJ31" s="1" t="str">
+        <v>BNP PARIBAS</v>
+      </c>
       <c r="AK31" s="1"/>
       <c r="AL31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
+      <c r="C32" s="1" t="str">
+        <v>BANK OF INDIA</v>
+      </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="str">
         <v>CNP／MASTERCARD 線上預授權</v>
@@ -14653,14 +14899,18 @@
       <c r="AG32" s="1"/>
       <c r="AH32" s="1"/>
       <c r="AI32" s="1"/>
-      <c r="AJ32" s="1"/>
+      <c r="AJ32" s="1" t="str">
+        <v>BANK OF INDIA</v>
+      </c>
       <c r="AK32" s="1"/>
       <c r="AL32" s="1"/>
     </row>
     <row r="33">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
+      <c r="C33" s="1" t="str">
+        <v>NATIONAL BANK OF PAKISTAN</v>
+      </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1" t="str">
         <v>CNP／DINERSCLUB 線上預授權</v>
@@ -14695,14 +14945,18 @@
       <c r="AG33" s="1"/>
       <c r="AH33" s="1"/>
       <c r="AI33" s="1"/>
-      <c r="AJ33" s="1"/>
+      <c r="AJ33" s="1" t="str">
+        <v>NATIONAL BANK OF PAKISTAN</v>
+      </c>
       <c r="AK33" s="1"/>
       <c r="AL33" s="1"/>
     </row>
     <row r="34">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
+      <c r="C34" s="1" t="str">
+        <v>大生銀行有限公司</v>
+      </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="str">
         <v>CNP／JCB 線上預授權</v>
@@ -14737,14 +14991,18 @@
       <c r="AG34" s="1"/>
       <c r="AH34" s="1"/>
       <c r="AI34" s="1"/>
-      <c r="AJ34" s="1"/>
+      <c r="AJ34" s="1" t="str">
+        <v>大生銀行有限公司</v>
+      </c>
       <c r="AK34" s="1"/>
       <c r="AL34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
+      <c r="C35" s="1" t="str">
+        <v>馬來亞銀行</v>
+      </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="str">
         <v>CNP／AMERICAEXPRESS 線上預授權</v>
@@ -14779,14 +15037,18 @@
       <c r="AG35" s="1"/>
       <c r="AH35" s="1"/>
       <c r="AI35" s="1"/>
-      <c r="AJ35" s="1"/>
+      <c r="AJ35" s="1" t="str">
+        <v>馬來亞銀行</v>
+      </c>
       <c r="AK35" s="1"/>
       <c r="AL35" s="1"/>
     </row>
     <row r="36">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
+      <c r="C36" s="1" t="str">
+        <v>SUMITOMO MITSUI BANKING CORPORATION</v>
+      </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1" t="str">
         <v>CNP／UNIONPAY 線上預授權</v>
@@ -14821,14 +15083,18 @@
       <c r="AG36" s="1"/>
       <c r="AH36" s="1"/>
       <c r="AI36" s="1"/>
-      <c r="AJ36" s="1"/>
+      <c r="AJ36" s="1" t="str">
+        <v>SUMITOMO MITSUI BANKING CORPORATION</v>
+      </c>
       <c r="AK36" s="1"/>
       <c r="AL36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
+      <c r="C37" s="1" t="str">
+        <v>PT. BANK NEGARA INDONESIA (PERSERO) TBK.</v>
+      </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="str">
         <v>CNP／UNIONPAY SecurePay</v>
@@ -14863,14 +15129,18 @@
       <c r="AG37" s="1"/>
       <c r="AH37" s="1"/>
       <c r="AI37" s="1"/>
-      <c r="AJ37" s="1"/>
+      <c r="AJ37" s="1" t="str">
+        <v>PT. BANK NEGARA INDONESIA (PERSERO) TBK.</v>
+      </c>
       <c r="AK37" s="1"/>
       <c r="AL37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
+      <c r="C38" s="1" t="str">
+        <v>金融銀行有限公司</v>
+      </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1" t="str">
         <v>CNP／VISA Click To Pay</v>
@@ -14905,14 +15175,18 @@
       <c r="AG38" s="1"/>
       <c r="AH38" s="1"/>
       <c r="AI38" s="1"/>
-      <c r="AJ38" s="1"/>
+      <c r="AJ38" s="1" t="str">
+        <v>金融銀行有限公司</v>
+      </c>
       <c r="AK38" s="1"/>
       <c r="AL38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
+      <c r="C39" s="1" t="str">
+        <v>大華銀行有限公司</v>
+      </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1" t="str">
         <v>CNP／MASTERCARD Click To Pay</v>
@@ -14947,14 +15221,18 @@
       <c r="AG39" s="1"/>
       <c r="AH39" s="1"/>
       <c r="AI39" s="1"/>
-      <c r="AJ39" s="1"/>
+      <c r="AJ39" s="1" t="str">
+        <v>大華銀行有限公司</v>
+      </c>
       <c r="AK39" s="1"/>
       <c r="AL39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
+      <c r="C40" s="1" t="str">
+        <v>中國工商銀行(亞洲)有限公司</v>
+      </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="str">
         <v>CNP／VISA Apple Pay</v>
@@ -14989,14 +15267,18 @@
       <c r="AG40" s="1"/>
       <c r="AH40" s="1"/>
       <c r="AI40" s="1"/>
-      <c r="AJ40" s="1"/>
+      <c r="AJ40" s="1" t="str">
+        <v>中國工商銀行(亞洲)有限公司</v>
+      </c>
       <c r="AK40" s="1"/>
       <c r="AL40" s="1"/>
     </row>
     <row r="41">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
+      <c r="C41" s="1" t="str">
+        <v>BARCLAYS BANK PLC.</v>
+      </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="str">
         <v>CNP／MASTERCARD Apple Pay</v>
@@ -15031,14 +15313,18 @@
       <c r="AG41" s="1"/>
       <c r="AH41" s="1"/>
       <c r="AI41" s="1"/>
-      <c r="AJ41" s="1"/>
+      <c r="AJ41" s="1" t="str">
+        <v>BARCLAYS BANK PLC.</v>
+      </c>
       <c r="AK41" s="1"/>
       <c r="AL41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
+      <c r="C42" s="1" t="str">
+        <v>THE BANK OF NOVA SCOTIA</v>
+      </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1" t="str">
         <v>CNP／VISA Google Pay</v>
@@ -15073,14 +15359,18 @@
       <c r="AG42" s="1"/>
       <c r="AH42" s="1"/>
       <c r="AI42" s="1"/>
-      <c r="AJ42" s="1"/>
+      <c r="AJ42" s="1" t="str">
+        <v>THE BANK OF NOVA SCOTIA</v>
+      </c>
       <c r="AK42" s="1"/>
       <c r="AL42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
+      <c r="C43" s="1" t="str">
+        <v>加拿大皇家銀行</v>
+      </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1" t="str">
         <v>CNP／MASTERCARD Google Pay</v>
@@ -15115,14 +15405,18 @@
       <c r="AG43" s="1"/>
       <c r="AH43" s="1"/>
       <c r="AI43" s="1"/>
-      <c r="AJ43" s="1"/>
+      <c r="AJ43" s="1" t="str">
+        <v>加拿大皇家銀行</v>
+      </c>
       <c r="AK43" s="1"/>
       <c r="AL43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
+      <c r="C44" s="1" t="str">
+        <v>法國興業銀行</v>
+      </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="str">
         <v>VisaDirect／VISA 本地付款</v>
@@ -15157,14 +15451,18 @@
       <c r="AG44" s="1"/>
       <c r="AH44" s="1"/>
       <c r="AI44" s="1"/>
-      <c r="AJ44" s="1"/>
+      <c r="AJ44" s="1" t="str">
+        <v>法國興業銀行</v>
+      </c>
       <c r="AK44" s="1"/>
       <c r="AL44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
+      <c r="C45" s="1" t="str">
+        <v>STATE BANK OF INDIA</v>
+      </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1" t="str">
         <v>VisaDirect／VISA 跨境實時付款</v>
@@ -15199,14 +15497,18 @@
       <c r="AG45" s="1"/>
       <c r="AH45" s="1"/>
       <c r="AI45" s="1"/>
-      <c r="AJ45" s="1"/>
+      <c r="AJ45" s="1" t="str">
+        <v>STATE BANK OF INDIA</v>
+      </c>
       <c r="AK45" s="1"/>
       <c r="AL45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
+      <c r="C46" s="1" t="str">
+        <v>多倫多道明銀行</v>
+      </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="str">
         <v>VisaDirect／VISA 跨境普通匯款</v>
@@ -15241,14 +15543,18 @@
       <c r="AG46" s="1"/>
       <c r="AH46" s="1"/>
       <c r="AI46" s="1"/>
-      <c r="AJ46" s="1"/>
+      <c r="AJ46" s="1" t="str">
+        <v>多倫多道明銀行</v>
+      </c>
       <c r="AK46" s="1"/>
       <c r="AL46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
+      <c r="C47" s="1" t="str">
+        <v>BANK OF MONTREAL</v>
+      </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1" t="str">
         <v>線上掃碼支付／微信掃碼-正掃</v>
@@ -15283,14 +15589,18 @@
       <c r="AG47" s="1"/>
       <c r="AH47" s="1"/>
       <c r="AI47" s="1"/>
-      <c r="AJ47" s="1"/>
+      <c r="AJ47" s="1" t="str">
+        <v>BANK OF MONTREAL</v>
+      </c>
       <c r="AK47" s="1"/>
       <c r="AL47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
+      <c r="C48" s="1" t="str">
+        <v>加拿大帝國商業銀行</v>
+      </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="str">
         <v>線上掃碼支付／微信APP支付</v>
@@ -15325,14 +15635,18 @@
       <c r="AG48" s="1"/>
       <c r="AH48" s="1"/>
       <c r="AI48" s="1"/>
-      <c r="AJ48" s="1"/>
+      <c r="AJ48" s="1" t="str">
+        <v>加拿大帝國商業銀行</v>
+      </c>
       <c r="AK48" s="1"/>
       <c r="AL48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
+      <c r="C49" s="1" t="str">
+        <v>UBS AG, HONG KONG</v>
+      </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1" t="str">
         <v>線上掃碼支付／微信小程序支付</v>
@@ -15367,14 +15681,18 @@
       <c r="AG49" s="1"/>
       <c r="AH49" s="1"/>
       <c r="AI49" s="1"/>
-      <c r="AJ49" s="1"/>
+      <c r="AJ49" s="1" t="str">
+        <v>UBS AG, HONG KONG</v>
+      </c>
       <c r="AK49" s="1"/>
       <c r="AL49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
+      <c r="C50" s="1" t="str">
+        <v>美國滙豐銀行</v>
+      </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1" t="str">
         <v>線上掃碼支付／微信公衆號支付</v>
@@ -15409,14 +15727,18 @@
       <c r="AG50" s="1"/>
       <c r="AH50" s="1"/>
       <c r="AI50" s="1"/>
-      <c r="AJ50" s="1"/>
+      <c r="AJ50" s="1" t="str">
+        <v>美國滙豐銀行</v>
+      </c>
       <c r="AK50" s="1"/>
       <c r="AL50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
+      <c r="C51" s="1" t="str">
+        <v>MIZUHO BANK, LTD.</v>
+      </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1" t="str">
         <v>線上掃碼支付／微信公衆號-服務商授權</v>
@@ -15451,14 +15773,18 @@
       <c r="AG51" s="1"/>
       <c r="AH51" s="1"/>
       <c r="AI51" s="1"/>
-      <c r="AJ51" s="1"/>
+      <c r="AJ51" s="1" t="str">
+        <v>MIZUHO BANK, LTD.</v>
+      </c>
       <c r="AK51" s="1"/>
       <c r="AL51" s="1"/>
     </row>
     <row r="52">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
+      <c r="C52" s="1" t="str">
+        <v>DZ BANK AG DEUTSCHE ZENTRAL- GENOSSENSCHAFTSBANK</v>
+      </c>
       <c r="D52" s="1"/>
       <c r="E52" s="1" t="str">
         <v>線上掃碼支付／微信H5支付</v>
@@ -15493,14 +15819,18 @@
       <c r="AG52" s="1"/>
       <c r="AH52" s="1"/>
       <c r="AI52" s="1"/>
-      <c r="AJ52" s="1"/>
+      <c r="AJ52" s="1" t="str">
+        <v>DZ BANK AG DEUTSCHE ZENTRAL- GENOSSENSCHAFTSBANK</v>
+      </c>
       <c r="AK52" s="1"/>
       <c r="AL52" s="1"/>
     </row>
     <row r="53">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
+      <c r="C53" s="1" t="str">
+        <v>友利銀行</v>
+      </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1" t="str">
         <v>線上掃碼支付／微信H5支付-服務商收銀台</v>
@@ -15535,14 +15865,18 @@
       <c r="AG53" s="1"/>
       <c r="AH53" s="1"/>
       <c r="AI53" s="1"/>
-      <c r="AJ53" s="1"/>
+      <c r="AJ53" s="1" t="str">
+        <v>友利銀行</v>
+      </c>
       <c r="AK53" s="1"/>
       <c r="AL53" s="1"/>
     </row>
     <row r="54">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
+      <c r="C54" s="1" t="str">
+        <v>PHILIPPINE NATIONAL BANK</v>
+      </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1" t="str">
         <v>線上掃碼支付／支付寶H5支付</v>
@@ -15577,14 +15911,18 @@
       <c r="AG54" s="1"/>
       <c r="AH54" s="1"/>
       <c r="AI54" s="1"/>
-      <c r="AJ54" s="1"/>
+      <c r="AJ54" s="1" t="str">
+        <v>PHILIPPINE NATIONAL BANK</v>
+      </c>
       <c r="AK54" s="1"/>
       <c r="AL54" s="1"/>
     </row>
     <row r="55">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
+      <c r="C55" s="1" t="str">
+        <v>富邦銀行(香港)有限公司</v>
+      </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1" t="str">
         <v>線上掃碼支付／支付寶APP支付</v>
@@ -15619,14 +15957,18 @@
       <c r="AG55" s="1"/>
       <c r="AH55" s="1"/>
       <c r="AI55" s="1"/>
-      <c r="AJ55" s="1"/>
+      <c r="AJ55" s="1" t="str">
+        <v>富邦銀行(香港)有限公司</v>
+      </c>
       <c r="AK55" s="1"/>
       <c r="AL55" s="1"/>
     </row>
     <row r="56">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
+      <c r="C56" s="1" t="str">
+        <v>MITSUBISHI UFJ TRUST AND BANKING CORPORATION</v>
+      </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1" t="str">
         <v>線上掃碼支付／支付寶WEB支付</v>
@@ -15661,14 +16003,18 @@
       <c r="AG56" s="1"/>
       <c r="AH56" s="1"/>
       <c r="AI56" s="1"/>
-      <c r="AJ56" s="1"/>
+      <c r="AJ56" s="1" t="str">
+        <v>MITSUBISHI UFJ TRUST AND BANKING CORPORATION</v>
+      </c>
       <c r="AK56" s="1"/>
       <c r="AL56" s="1"/>
     </row>
     <row r="57">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
+      <c r="C57" s="1" t="str">
+        <v>THE BANK OF NEW YORK MELLON</v>
+      </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1" t="str">
         <v>線上掃碼支付／銀聯雲閃付掃碼-正掃</v>
@@ -15703,14 +16049,18 @@
       <c r="AG57" s="1"/>
       <c r="AH57" s="1"/>
       <c r="AI57" s="1"/>
-      <c r="AJ57" s="1"/>
+      <c r="AJ57" s="1" t="str">
+        <v>THE BANK OF NEW YORK MELLON</v>
+      </c>
       <c r="AK57" s="1"/>
       <c r="AL57" s="1"/>
     </row>
     <row r="58">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
+      <c r="C58" s="1" t="str">
+        <v>ING BANK N.V.</v>
+      </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1" t="str">
         <v>線上掃碼支付／payNow-正掃</v>
@@ -15745,14 +16095,18 @@
       <c r="AG58" s="1"/>
       <c r="AH58" s="1"/>
       <c r="AI58" s="1"/>
-      <c r="AJ58" s="1"/>
+      <c r="AJ58" s="1" t="str">
+        <v>ING BANK N.V.</v>
+      </c>
       <c r="AK58" s="1"/>
       <c r="AL58" s="1"/>
     </row>
     <row r="59">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
+      <c r="C59" s="1" t="str">
+        <v>BANCO BILBAO VIZCAYA ARGENTARIA, S.A.</v>
+      </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1" t="str">
         <v>線上掃碼支付／八達通-正掃</v>
@@ -15787,14 +16141,18 @@
       <c r="AG59" s="1"/>
       <c r="AH59" s="1"/>
       <c r="AI59" s="1"/>
-      <c r="AJ59" s="1"/>
+      <c r="AJ59" s="1" t="str">
+        <v>BANCO BILBAO VIZCAYA ARGENTARIA, S.A.</v>
+      </c>
       <c r="AK59" s="1"/>
       <c r="AL59" s="1"/>
     </row>
     <row r="60">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
+      <c r="C60" s="1" t="str">
+        <v>澳大利亞國民銀行</v>
+      </c>
       <c r="D60" s="1"/>
       <c r="E60" s="1" t="str">
         <v>線上掃碼支付／八達通-WEB支付</v>
@@ -15829,14 +16187,18 @@
       <c r="AG60" s="1"/>
       <c r="AH60" s="1"/>
       <c r="AI60" s="1"/>
-      <c r="AJ60" s="1"/>
+      <c r="AJ60" s="1" t="str">
+        <v>澳大利亞國民銀行</v>
+      </c>
       <c r="AK60" s="1"/>
       <c r="AL60" s="1"/>
     </row>
     <row r="61">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
+      <c r="C61" s="1" t="str">
+        <v>澳新銀行集團有限公司</v>
+      </c>
       <c r="D61" s="1"/>
       <c r="E61" s="1" t="str">
         <v>線下掃碼支付／微信掃碼-正掃</v>
@@ -15871,14 +16233,18 @@
       <c r="AG61" s="1"/>
       <c r="AH61" s="1"/>
       <c r="AI61" s="1"/>
-      <c r="AJ61" s="1"/>
+      <c r="AJ61" s="1" t="str">
+        <v>澳新銀行集團有限公司</v>
+      </c>
       <c r="AK61" s="1"/>
       <c r="AL61" s="1"/>
     </row>
     <row r="62">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
+      <c r="C62" s="1" t="str">
+        <v>澳洲聯邦銀行</v>
+      </c>
       <c r="D62" s="1"/>
       <c r="E62" s="1" t="str">
         <v>線下掃碼支付／微信刷卡-反掃</v>
@@ -15913,14 +16279,18 @@
       <c r="AG62" s="1"/>
       <c r="AH62" s="1"/>
       <c r="AI62" s="1"/>
-      <c r="AJ62" s="1"/>
+      <c r="AJ62" s="1" t="str">
+        <v>澳洲聯邦銀行</v>
+      </c>
       <c r="AK62" s="1"/>
       <c r="AL62" s="1"/>
     </row>
     <row r="63">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
-      <c r="C63" s="1"/>
+      <c r="C63" s="1" t="str">
+        <v>意大利聯合聖保羅銀行股份有限公司</v>
+      </c>
       <c r="D63" s="1"/>
       <c r="E63" s="1" t="str">
         <v>線下掃碼支付／微信公衆號支付</v>
@@ -15955,14 +16325,18 @@
       <c r="AG63" s="1"/>
       <c r="AH63" s="1"/>
       <c r="AI63" s="1"/>
-      <c r="AJ63" s="1"/>
+      <c r="AJ63" s="1" t="str">
+        <v>意大利聯合聖保羅銀行股份有限公司</v>
+      </c>
       <c r="AK63" s="1"/>
       <c r="AL63" s="1"/>
     </row>
     <row r="64">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
-      <c r="C64" s="1"/>
+      <c r="C64" s="1" t="str">
+        <v>裕信(德國)銀行股份有限公司</v>
+      </c>
       <c r="D64" s="1"/>
       <c r="E64" s="1" t="str">
         <v>線下掃碼支付／微信公衆號-服務商授權</v>
@@ -15997,14 +16371,18 @@
       <c r="AG64" s="1"/>
       <c r="AH64" s="1"/>
       <c r="AI64" s="1"/>
-      <c r="AJ64" s="1"/>
+      <c r="AJ64" s="1" t="str">
+        <v>裕信(德國)銀行股份有限公司</v>
+      </c>
       <c r="AK64" s="1"/>
       <c r="AL64" s="1"/>
     </row>
     <row r="65">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
-      <c r="C65" s="1"/>
+      <c r="C65" s="1" t="str">
+        <v>THE CHIBA BANK LTD</v>
+      </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1" t="str">
         <v>線下掃碼支付／支付寶-正掃</v>
@@ -16039,14 +16417,18 @@
       <c r="AG65" s="1"/>
       <c r="AH65" s="1"/>
       <c r="AI65" s="1"/>
-      <c r="AJ65" s="1"/>
+      <c r="AJ65" s="1" t="str">
+        <v>THE CHIBA BANK LTD</v>
+      </c>
       <c r="AK65" s="1"/>
       <c r="AL65" s="1"/>
     </row>
     <row r="66">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
-      <c r="C66" s="1"/>
+      <c r="C66" s="1" t="str">
+        <v>比利時聯合銀行</v>
+      </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1" t="str">
         <v>線下掃碼支付／支付寶刷卡-反掃</v>
@@ -16081,14 +16463,18 @@
       <c r="AG66" s="1"/>
       <c r="AH66" s="1"/>
       <c r="AI66" s="1"/>
-      <c r="AJ66" s="1"/>
+      <c r="AJ66" s="1" t="str">
+        <v>比利時聯合銀行</v>
+      </c>
       <c r="AK66" s="1"/>
       <c r="AL66" s="1"/>
     </row>
     <row r="67">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
-      <c r="C67" s="1"/>
+      <c r="C67" s="1" t="str">
+        <v>WELLS FARGO BANK, N.A.</v>
+      </c>
       <c r="D67" s="1"/>
       <c r="E67" s="1" t="str">
         <v>線下掃碼支付／銀聯雲閃付掃碼-正掃</v>
@@ -16123,14 +16509,18 @@
       <c r="AG67" s="1"/>
       <c r="AH67" s="1"/>
       <c r="AI67" s="1"/>
-      <c r="AJ67" s="1"/>
+      <c r="AJ67" s="1" t="str">
+        <v>WELLS FARGO BANK, N.A.</v>
+      </c>
       <c r="AK67" s="1"/>
       <c r="AL67" s="1"/>
     </row>
     <row r="68">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
-      <c r="C68" s="1"/>
+      <c r="C68" s="1" t="str">
+        <v>COÖPERATIEVE RABOBANK U.A.</v>
+      </c>
       <c r="D68" s="1"/>
       <c r="E68" s="1" t="str">
         <v>線下掃碼支付／銀聯雲閃付刷卡-反掃</v>
@@ -16165,14 +16555,18 @@
       <c r="AG68" s="1"/>
       <c r="AH68" s="1"/>
       <c r="AI68" s="1"/>
-      <c r="AJ68" s="1"/>
+      <c r="AJ68" s="1" t="str">
+        <v>COÖPERATIEVE RABOBANK U.A.</v>
+      </c>
       <c r="AK68" s="1"/>
       <c r="AL68" s="1"/>
     </row>
     <row r="69">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
-      <c r="C69" s="1"/>
+      <c r="C69" s="1" t="str">
+        <v>DBS BANK LTD, HONG KONG BRANCH</v>
+      </c>
       <c r="D69" s="1"/>
       <c r="E69" s="1" t="str">
         <v>線下掃碼支付／payNow-正掃</v>
@@ -16207,14 +16601,18 @@
       <c r="AG69" s="1"/>
       <c r="AH69" s="1"/>
       <c r="AI69" s="1"/>
-      <c r="AJ69" s="1"/>
+      <c r="AJ69" s="1" t="str">
+        <v>DBS BANK LTD, HONG KONG BRANCH</v>
+      </c>
       <c r="AK69" s="1"/>
       <c r="AL69" s="1"/>
     </row>
     <row r="70">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
-      <c r="C70" s="1"/>
+      <c r="C70" s="1" t="str">
+        <v>靜岡銀行</v>
+      </c>
       <c r="D70" s="1"/>
       <c r="E70" s="1" t="str">
         <v>線下掃碼支付／PayMe掃碼-正掃</v>
@@ -16249,14 +16647,18 @@
       <c r="AG70" s="1"/>
       <c r="AH70" s="1"/>
       <c r="AI70" s="1"/>
-      <c r="AJ70" s="1"/>
+      <c r="AJ70" s="1" t="str">
+        <v>靜岡銀行</v>
+      </c>
       <c r="AK70" s="1"/>
       <c r="AL70" s="1"/>
     </row>
     <row r="71">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
+      <c r="C71" s="1" t="str">
+        <v>華南商業銀行股份有限公司</v>
+      </c>
       <c r="D71" s="1"/>
       <c r="E71" s="1" t="str">
         <v>線下掃碼支付／PayMe刷卡-反掃</v>
@@ -16291,14 +16693,18 @@
       <c r="AG71" s="1"/>
       <c r="AH71" s="1"/>
       <c r="AI71" s="1"/>
-      <c r="AJ71" s="1"/>
+      <c r="AJ71" s="1" t="str">
+        <v>華南商業銀行股份有限公司</v>
+      </c>
       <c r="AK71" s="1"/>
       <c r="AL71" s="1"/>
     </row>
     <row r="72">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
+      <c r="C72" s="1" t="str">
+        <v>THE SHIGA BANK, LTD.</v>
+      </c>
       <c r="D72" s="1"/>
       <c r="E72" s="1" t="str">
         <v>線下掃碼支付／八達通-正掃</v>
@@ -16333,14 +16739,18 @@
       <c r="AG72" s="1"/>
       <c r="AH72" s="1"/>
       <c r="AI72" s="1"/>
-      <c r="AJ72" s="1"/>
+      <c r="AJ72" s="1" t="str">
+        <v>THE SHIGA BANK, LTD.</v>
+      </c>
       <c r="AK72" s="1"/>
       <c r="AL72" s="1"/>
     </row>
     <row r="73">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
-      <c r="C73" s="1"/>
+      <c r="C73" s="1" t="str">
+        <v>臺灣銀行股份有限公司</v>
+      </c>
       <c r="D73" s="1"/>
       <c r="E73" s="1" t="str">
         <v>PayByLink／微信掃碼-正掃</v>
@@ -16375,14 +16785,18 @@
       <c r="AG73" s="1"/>
       <c r="AH73" s="1"/>
       <c r="AI73" s="1"/>
-      <c r="AJ73" s="1"/>
+      <c r="AJ73" s="1" t="str">
+        <v>臺灣銀行股份有限公司</v>
+      </c>
       <c r="AK73" s="1"/>
       <c r="AL73" s="1"/>
     </row>
     <row r="74">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
-      <c r="C74" s="1"/>
+      <c r="C74" s="1" t="str">
+        <v>THE CHUGOKU BANK LIMITED</v>
+      </c>
       <c r="D74" s="1"/>
       <c r="E74" s="1" t="str">
         <v>PayByLink／微信H5支付-服務商收銀台</v>
@@ -16417,14 +16831,18 @@
       <c r="AG74" s="1"/>
       <c r="AH74" s="1"/>
       <c r="AI74" s="1"/>
-      <c r="AJ74" s="1"/>
+      <c r="AJ74" s="1" t="str">
+        <v>THE CHUGOKU BANK LIMITED</v>
+      </c>
       <c r="AK74" s="1"/>
       <c r="AL74" s="1"/>
     </row>
     <row r="75">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
+      <c r="C75" s="1" t="str">
+        <v>第一商業銀行股份有限公司</v>
+      </c>
       <c r="D75" s="1"/>
       <c r="E75" s="1" t="str">
         <v>PayByLink／微信公衆號-服務商授權</v>
@@ -16459,14 +16877,18 @@
       <c r="AG75" s="1"/>
       <c r="AH75" s="1"/>
       <c r="AI75" s="1"/>
-      <c r="AJ75" s="1"/>
+      <c r="AJ75" s="1" t="str">
+        <v>第一商業銀行股份有限公司</v>
+      </c>
       <c r="AK75" s="1"/>
       <c r="AL75" s="1"/>
     </row>
     <row r="76">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
-      <c r="C76" s="1"/>
+      <c r="C76" s="1" t="str">
+        <v>彰化商業銀行股份有限公司</v>
+      </c>
       <c r="D76" s="1"/>
       <c r="E76" s="1" t="str">
         <v>PayByLink／支付寶H5支付</v>
@@ -16501,14 +16923,18 @@
       <c r="AG76" s="1"/>
       <c r="AH76" s="1"/>
       <c r="AI76" s="1"/>
-      <c r="AJ76" s="1"/>
+      <c r="AJ76" s="1" t="str">
+        <v>彰化商業銀行股份有限公司</v>
+      </c>
       <c r="AK76" s="1"/>
       <c r="AL76" s="1"/>
     </row>
     <row r="77">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
-      <c r="C77" s="1"/>
+      <c r="C77" s="1" t="str">
+        <v>NATIXIS</v>
+      </c>
       <c r="D77" s="1"/>
       <c r="E77" s="1" t="str">
         <v>PayByLink／支付寶WEB支付</v>
@@ -16543,14 +16969,18 @@
       <c r="AG77" s="1"/>
       <c r="AH77" s="1"/>
       <c r="AI77" s="1"/>
-      <c r="AJ77" s="1"/>
+      <c r="AJ77" s="1" t="str">
+        <v>NATIXIS</v>
+      </c>
       <c r="AK77" s="1"/>
       <c r="AL77" s="1"/>
     </row>
     <row r="78">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
+      <c r="C78" s="1" t="str">
+        <v>中國工商銀行股份有限公司</v>
+      </c>
       <c r="D78" s="1"/>
       <c r="E78" s="1" t="str">
         <v>PayByLink／銀聯雲閃付掃碼-正掃</v>
@@ -16585,14 +17015,18 @@
       <c r="AG78" s="1"/>
       <c r="AH78" s="1"/>
       <c r="AI78" s="1"/>
-      <c r="AJ78" s="1"/>
+      <c r="AJ78" s="1" t="str">
+        <v>中國工商銀行股份有限公司</v>
+      </c>
       <c r="AK78" s="1"/>
       <c r="AL78" s="1"/>
     </row>
     <row r="79">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="1"/>
+      <c r="C79" s="1" t="str">
+        <v>STATE STREET BANK AND TRUST COMPANY</v>
+      </c>
       <c r="D79" s="1"/>
       <c r="E79" s="1" t="str">
         <v>PayByLink／payNow-正掃</v>
@@ -16627,14 +17061,18 @@
       <c r="AG79" s="1"/>
       <c r="AH79" s="1"/>
       <c r="AI79" s="1"/>
-      <c r="AJ79" s="1"/>
+      <c r="AJ79" s="1" t="str">
+        <v>STATE STREET BANK AND TRUST COMPANY</v>
+      </c>
       <c r="AK79" s="1"/>
       <c r="AL79" s="1"/>
     </row>
     <row r="80">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
-      <c r="C80" s="1"/>
+      <c r="C80" s="1" t="str">
+        <v>中國建設銀行股份有限公司</v>
+      </c>
       <c r="D80" s="1"/>
       <c r="E80" s="1" t="str">
         <v>PayByLink／八達通-正掃</v>
@@ -16669,14 +17107,18 @@
       <c r="AG80" s="1"/>
       <c r="AH80" s="1"/>
       <c r="AI80" s="1"/>
-      <c r="AJ80" s="1"/>
+      <c r="AJ80" s="1" t="str">
+        <v>中國建設銀行股份有限公司</v>
+      </c>
       <c r="AK80" s="1"/>
       <c r="AL80" s="1"/>
     </row>
     <row r="81">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
-      <c r="C81" s="1"/>
+      <c r="C81" s="1" t="str">
+        <v>中國農業銀行股份有限公司</v>
+      </c>
       <c r="D81" s="1"/>
       <c r="E81" s="1" t="str">
         <v>PayByLink／八達通-WEB支付</v>
@@ -16711,14 +17153,18 @@
       <c r="AG81" s="1"/>
       <c r="AH81" s="1"/>
       <c r="AI81" s="1"/>
-      <c r="AJ81" s="1"/>
+      <c r="AJ81" s="1" t="str">
+        <v>中國農業銀行股份有限公司</v>
+      </c>
       <c r="AK81" s="1"/>
       <c r="AL81" s="1"/>
     </row>
     <row r="82">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
+      <c r="C82" s="1" t="str">
+        <v>ERSTE GROUP BANK AG</v>
+      </c>
       <c r="D82" s="1"/>
       <c r="E82" s="1" t="str">
         <v>PayByLink／VISA 線上消費</v>
@@ -16753,14 +17199,18 @@
       <c r="AG82" s="1"/>
       <c r="AH82" s="1"/>
       <c r="AI82" s="1"/>
-      <c r="AJ82" s="1"/>
+      <c r="AJ82" s="1" t="str">
+        <v>ERSTE GROUP BANK AG</v>
+      </c>
       <c r="AK82" s="1"/>
       <c r="AL82" s="1"/>
     </row>
     <row r="83">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
+      <c r="C83" s="1" t="str">
+        <v>中國信託商業銀行股份有限公司</v>
+      </c>
       <c r="D83" s="1"/>
       <c r="E83" s="1" t="str">
         <v>PayByLink／MASTERCARD 線上消費</v>
@@ -16795,14 +17245,18 @@
       <c r="AG83" s="1"/>
       <c r="AH83" s="1"/>
       <c r="AI83" s="1"/>
-      <c r="AJ83" s="1"/>
+      <c r="AJ83" s="1" t="str">
+        <v>中國信託商業銀行股份有限公司</v>
+      </c>
       <c r="AK83" s="1"/>
       <c r="AL83" s="1"/>
     </row>
     <row r="84">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
-      <c r="C84" s="1"/>
+      <c r="C84" s="1" t="str">
+        <v>臺灣中小企業銀行股份有限公司</v>
+      </c>
       <c r="D84" s="1"/>
       <c r="E84" s="1" t="str">
         <v>PayByLink／JCB 線上消費</v>
@@ -16837,14 +17291,18 @@
       <c r="AG84" s="1"/>
       <c r="AH84" s="1"/>
       <c r="AI84" s="1"/>
-      <c r="AJ84" s="1"/>
+      <c r="AJ84" s="1" t="str">
+        <v>臺灣中小企業銀行股份有限公司</v>
+      </c>
       <c r="AK84" s="1"/>
       <c r="AL84" s="1"/>
     </row>
     <row r="85">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
-      <c r="C85" s="1"/>
+      <c r="C85" s="1" t="str">
+        <v>國泰世華商業銀行股份有限公司</v>
+      </c>
       <c r="D85" s="1"/>
       <c r="E85" s="1" t="str">
         <v>PayByLink／AMERICAEXPRESS 線上消費</v>
@@ -16879,14 +17337,18 @@
       <c r="AG85" s="1"/>
       <c r="AH85" s="1"/>
       <c r="AI85" s="1"/>
-      <c r="AJ85" s="1"/>
+      <c r="AJ85" s="1" t="str">
+        <v>國泰世華商業銀行股份有限公司</v>
+      </c>
       <c r="AK85" s="1"/>
       <c r="AL85" s="1"/>
     </row>
     <row r="86">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
-      <c r="C86" s="1"/>
+      <c r="C86" s="1" t="str">
+        <v>瑞士盈豐銀行股份有限公司</v>
+      </c>
       <c r="D86" s="1"/>
       <c r="E86" s="1" t="str">
         <v>PayByLink／UNIONPAY 線上消費</v>
@@ -16921,14 +17383,18 @@
       <c r="AG86" s="1"/>
       <c r="AH86" s="1"/>
       <c r="AI86" s="1"/>
-      <c r="AJ86" s="1"/>
+      <c r="AJ86" s="1" t="str">
+        <v>瑞士盈豐銀行股份有限公司</v>
+      </c>
       <c r="AK86" s="1"/>
       <c r="AL86" s="1"/>
     </row>
     <row r="87">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
-      <c r="C87" s="1"/>
+      <c r="C87" s="1" t="str">
+        <v>招商銀行股份有限公司</v>
+      </c>
       <c r="D87" s="1"/>
       <c r="E87" s="1" t="str">
         <v>PayByLink／UNIONPAY SecurePay</v>
@@ -16963,14 +17429,18 @@
       <c r="AG87" s="1"/>
       <c r="AH87" s="1"/>
       <c r="AI87" s="1"/>
-      <c r="AJ87" s="1"/>
+      <c r="AJ87" s="1" t="str">
+        <v>招商銀行股份有限公司</v>
+      </c>
       <c r="AK87" s="1"/>
       <c r="AL87" s="1"/>
     </row>
     <row r="88">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
-      <c r="C88" s="1"/>
+      <c r="C88" s="1" t="str">
+        <v>台北富邦商業銀行股份有限公司</v>
+      </c>
       <c r="D88" s="1"/>
       <c r="E88" s="1" t="str">
         <v>PayByLink／VISA Click To Pay</v>
@@ -17005,14 +17475,18 @@
       <c r="AG88" s="1"/>
       <c r="AH88" s="1"/>
       <c r="AI88" s="1"/>
-      <c r="AJ88" s="1"/>
+      <c r="AJ88" s="1" t="str">
+        <v>台北富邦商業銀行股份有限公司</v>
+      </c>
       <c r="AK88" s="1"/>
       <c r="AL88" s="1"/>
     </row>
     <row r="89">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
-      <c r="C89" s="1"/>
+      <c r="C89" s="1" t="str">
+        <v>永豐商業銀行股份有限公司</v>
+      </c>
       <c r="D89" s="1"/>
       <c r="E89" s="1" t="str">
         <v>PayByLink／MASTERCARD Click To Pay</v>
@@ -17047,14 +17521,18 @@
       <c r="AG89" s="1"/>
       <c r="AH89" s="1"/>
       <c r="AI89" s="1"/>
-      <c r="AJ89" s="1"/>
+      <c r="AJ89" s="1" t="str">
+        <v>永豐商業銀行股份有限公司</v>
+      </c>
       <c r="AK89" s="1"/>
       <c r="AL89" s="1"/>
     </row>
     <row r="90">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
-      <c r="C90" s="1"/>
+      <c r="C90" s="1" t="str">
+        <v>兆豐國際商業銀行股份有限公司</v>
+      </c>
       <c r="D90" s="1"/>
       <c r="E90" s="1" t="str">
         <v>PayByLink／VISA Apple Pay</v>
@@ -17089,14 +17567,18 @@
       <c r="AG90" s="1"/>
       <c r="AH90" s="1"/>
       <c r="AI90" s="1"/>
-      <c r="AJ90" s="1"/>
+      <c r="AJ90" s="1" t="str">
+        <v>兆豐國際商業銀行股份有限公司</v>
+      </c>
       <c r="AK90" s="1"/>
       <c r="AL90" s="1"/>
     </row>
     <row r="91">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
-      <c r="C91" s="1"/>
+      <c r="C91" s="1" t="str">
+        <v>玉山商業銀行股份有限公司</v>
+      </c>
       <c r="D91" s="1"/>
       <c r="E91" s="1" t="str">
         <v>PayByLink／MASTERCARD Apple Pay</v>
@@ -17131,14 +17613,18 @@
       <c r="AG91" s="1"/>
       <c r="AH91" s="1"/>
       <c r="AI91" s="1"/>
-      <c r="AJ91" s="1"/>
+      <c r="AJ91" s="1" t="str">
+        <v>玉山商業銀行股份有限公司</v>
+      </c>
       <c r="AK91" s="1"/>
       <c r="AL91" s="1"/>
     </row>
     <row r="92">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
-      <c r="C92" s="1"/>
+      <c r="C92" s="1" t="str">
+        <v>台新國際商業銀行股份有限公司</v>
+      </c>
       <c r="D92" s="1"/>
       <c r="E92" s="1" t="str">
         <v>PayByLink／VISA Google Pay</v>
@@ -17173,14 +17659,18 @@
       <c r="AG92" s="1"/>
       <c r="AH92" s="1"/>
       <c r="AI92" s="1"/>
-      <c r="AJ92" s="1"/>
+      <c r="AJ92" s="1" t="str">
+        <v>台新國際商業銀行股份有限公司</v>
+      </c>
       <c r="AK92" s="1"/>
       <c r="AL92" s="1"/>
     </row>
     <row r="93">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
-      <c r="C93" s="1"/>
+      <c r="C93" s="1" t="str">
+        <v>豐隆銀行有限公司</v>
+      </c>
       <c r="D93" s="1"/>
       <c r="E93" s="1" t="str">
         <v>PayByLink／MASTERCARD Google Pay</v>
@@ -17215,14 +17705,18 @@
       <c r="AG93" s="1"/>
       <c r="AH93" s="1"/>
       <c r="AI93" s="1"/>
-      <c r="AJ93" s="1"/>
+      <c r="AJ93" s="1" t="str">
+        <v>豐隆銀行有限公司</v>
+      </c>
       <c r="AK93" s="1"/>
       <c r="AL93" s="1"/>
     </row>
     <row r="94">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
+      <c r="C94" s="1" t="str">
+        <v>渣打銀行</v>
+      </c>
       <c r="D94" s="1"/>
       <c r="E94" s="1" t="str">
         <v>帳戶驗證／VISA 賬戶驗證</v>
@@ -17257,14 +17751,18 @@
       <c r="AG94" s="1"/>
       <c r="AH94" s="1"/>
       <c r="AI94" s="1"/>
-      <c r="AJ94" s="1"/>
+      <c r="AJ94" s="1" t="str">
+        <v>渣打銀行</v>
+      </c>
       <c r="AK94" s="1"/>
       <c r="AL94" s="1"/>
     </row>
     <row r="95">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
+      <c r="C95" s="1" t="str">
+        <v>花旗銀行(香港)有限公司</v>
+      </c>
       <c r="D95" s="1"/>
       <c r="E95" s="1" t="str">
         <v>帳戶驗證／MASTERCARD 賬戶驗證</v>
@@ -17299,14 +17797,18 @@
       <c r="AG95" s="1"/>
       <c r="AH95" s="1"/>
       <c r="AI95" s="1"/>
-      <c r="AJ95" s="1"/>
+      <c r="AJ95" s="1" t="str">
+        <v>花旗銀行(香港)有限公司</v>
+      </c>
       <c r="AK95" s="1"/>
       <c r="AL95" s="1"/>
     </row>
     <row r="96">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
-      <c r="C96" s="1"/>
+      <c r="C96" s="1" t="str">
+        <v>ICICI BANK LIMITED</v>
+      </c>
       <c r="D96" s="1"/>
       <c r="E96" s="1" t="str">
         <v>帳戶驗證／UNIONPAY 帳戶風險篩查</v>
@@ -17341,14 +17843,18 @@
       <c r="AG96" s="1"/>
       <c r="AH96" s="1"/>
       <c r="AI96" s="1"/>
-      <c r="AJ96" s="1"/>
+      <c r="AJ96" s="1" t="str">
+        <v>ICICI BANK LIMITED</v>
+      </c>
       <c r="AK96" s="1"/>
       <c r="AL96" s="1"/>
     </row>
     <row r="97">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
-      <c r="C97" s="1"/>
+      <c r="C97" s="1" t="str">
+        <v>MELLI BANK PLC</v>
+      </c>
       <c r="D97" s="1"/>
       <c r="E97" s="1" t="str">
         <v>增值服務／微信報關</v>
@@ -17383,14 +17889,18 @@
       <c r="AG97" s="1"/>
       <c r="AH97" s="1"/>
       <c r="AI97" s="1"/>
-      <c r="AJ97" s="1"/>
+      <c r="AJ97" s="1" t="str">
+        <v>MELLI BANK PLC</v>
+      </c>
       <c r="AK97" s="1"/>
       <c r="AL97" s="1"/>
     </row>
     <row r="98">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
+      <c r="C98" s="1" t="str">
+        <v>華美銀行</v>
+      </c>
       <c r="D98" s="1"/>
       <c r="E98" s="1" t="str">
         <v>一碼付／微信H5支付-服務商收銀台</v>
@@ -17425,14 +17935,18 @@
       <c r="AG98" s="1"/>
       <c r="AH98" s="1"/>
       <c r="AI98" s="1"/>
-      <c r="AJ98" s="1"/>
+      <c r="AJ98" s="1" t="str">
+        <v>華美銀行</v>
+      </c>
       <c r="AK98" s="1"/>
       <c r="AL98" s="1"/>
     </row>
     <row r="99">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
+      <c r="C99" s="1" t="str">
+        <v>遠東國際商業銀行股份有限公司</v>
+      </c>
       <c r="D99" s="1"/>
       <c r="E99" s="1" t="str">
         <v>一碼付／微信公衆號-服務商授權</v>
@@ -17467,14 +17981,18 @@
       <c r="AG99" s="1"/>
       <c r="AH99" s="1"/>
       <c r="AI99" s="1"/>
-      <c r="AJ99" s="1"/>
+      <c r="AJ99" s="1" t="str">
+        <v>遠東國際商業銀行股份有限公司</v>
+      </c>
       <c r="AK99" s="1"/>
       <c r="AL99" s="1"/>
     </row>
     <row r="100">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
-      <c r="C100" s="1"/>
+      <c r="C100" s="1" t="str">
+        <v>國泰銀行</v>
+      </c>
       <c r="D100" s="1"/>
       <c r="E100" s="1" t="str">
         <v>一碼付／支付寶H5支付</v>
@@ -17509,14 +18027,18 @@
       <c r="AG100" s="1"/>
       <c r="AH100" s="1"/>
       <c r="AI100" s="1"/>
-      <c r="AJ100" s="1"/>
+      <c r="AJ100" s="1" t="str">
+        <v>國泰銀行</v>
+      </c>
       <c r="AK100" s="1"/>
       <c r="AL100" s="1"/>
     </row>
     <row r="101">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
+      <c r="C101" s="1" t="str">
+        <v>臺灣土地銀行股份有限公司</v>
+      </c>
       <c r="D101" s="1"/>
       <c r="E101" s="1" t="str">
         <v>一碼付／支付寶-正掃</v>
@@ -17551,14 +18073,18 @@
       <c r="AG101" s="1"/>
       <c r="AH101" s="1"/>
       <c r="AI101" s="1"/>
-      <c r="AJ101" s="1"/>
+      <c r="AJ101" s="1" t="str">
+        <v>臺灣土地銀行股份有限公司</v>
+      </c>
       <c r="AK101" s="1"/>
       <c r="AL101" s="1"/>
     </row>
     <row r="102">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
-      <c r="C102" s="1"/>
+      <c r="C102" s="1" t="str">
+        <v>合作金庫商業銀行股份有限公司</v>
+      </c>
       <c r="D102" s="1"/>
       <c r="E102" s="1" t="str">
         <v>一碼付／payNow-正掃</v>
@@ -17593,14 +18119,18 @@
       <c r="AG102" s="1"/>
       <c r="AH102" s="1"/>
       <c r="AI102" s="1"/>
-      <c r="AJ102" s="1"/>
+      <c r="AJ102" s="1" t="str">
+        <v>合作金庫商業銀行股份有限公司</v>
+      </c>
       <c r="AK102" s="1"/>
       <c r="AL102" s="1"/>
     </row>
     <row r="103">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
-      <c r="C103" s="1"/>
+      <c r="C103" s="1" t="str">
+        <v>西班牙桑坦德銀行有限公司</v>
+      </c>
       <c r="D103" s="1"/>
       <c r="E103" s="1" t="str">
         <v>一碼付／八達通-WEB支付</v>
@@ -17635,14 +18165,18 @@
       <c r="AG103" s="1"/>
       <c r="AH103" s="1"/>
       <c r="AI103" s="1"/>
-      <c r="AJ103" s="1"/>
+      <c r="AJ103" s="1" t="str">
+        <v>西班牙桑坦德銀行有限公司</v>
+      </c>
       <c r="AK103" s="1"/>
       <c r="AL103" s="1"/>
     </row>
     <row r="104">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
-      <c r="C104" s="1"/>
+      <c r="C104" s="1" t="str">
+        <v>上海商業儲蓄銀行股份有限公司</v>
+      </c>
       <c r="D104" s="1"/>
       <c r="E104" s="1" t="str">
         <v>一碼付／VISA 線上消費</v>
@@ -17677,14 +18211,18 @@
       <c r="AG104" s="1"/>
       <c r="AH104" s="1"/>
       <c r="AI104" s="1"/>
-      <c r="AJ104" s="1"/>
+      <c r="AJ104" s="1" t="str">
+        <v>上海商業儲蓄銀行股份有限公司</v>
+      </c>
       <c r="AK104" s="1"/>
       <c r="AL104" s="1"/>
     </row>
     <row r="105">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
-      <c r="C105" s="1"/>
+      <c r="C105" s="1" t="str">
+        <v>INDUSTRIAL BANK OF KOREA</v>
+      </c>
       <c r="D105" s="1"/>
       <c r="E105" s="1" t="str">
         <v>一碼付／MASTERCARD 線上消費</v>
@@ -17719,14 +18257,18 @@
       <c r="AG105" s="1"/>
       <c r="AH105" s="1"/>
       <c r="AI105" s="1"/>
-      <c r="AJ105" s="1"/>
+      <c r="AJ105" s="1" t="str">
+        <v>INDUSTRIAL BANK OF KOREA</v>
+      </c>
       <c r="AK105" s="1"/>
       <c r="AL105" s="1"/>
     </row>
     <row r="106">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
-      <c r="C106" s="1"/>
+      <c r="C106" s="1" t="str">
+        <v>新加坡銀行有限公司</v>
+      </c>
       <c r="D106" s="1"/>
       <c r="E106" s="1" t="str">
         <v>一碼付／JCB 線上消費</v>
@@ -17761,14 +18303,18 @@
       <c r="AG106" s="1"/>
       <c r="AH106" s="1"/>
       <c r="AI106" s="1"/>
-      <c r="AJ106" s="1"/>
+      <c r="AJ106" s="1" t="str">
+        <v>新加坡銀行有限公司</v>
+      </c>
       <c r="AK106" s="1"/>
       <c r="AL106" s="1"/>
     </row>
     <row r="107">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
+      <c r="C107" s="1" t="str">
+        <v>SHINHAN BANK</v>
+      </c>
       <c r="D107" s="1"/>
       <c r="E107" s="1" t="str">
         <v>一碼付／AMERICAEXPRESS 線上消費</v>
@@ -17803,14 +18349,18 @@
       <c r="AG107" s="1"/>
       <c r="AH107" s="1"/>
       <c r="AI107" s="1"/>
-      <c r="AJ107" s="1"/>
+      <c r="AJ107" s="1" t="str">
+        <v>SHINHAN BANK</v>
+      </c>
       <c r="AK107" s="1"/>
       <c r="AL107" s="1"/>
     </row>
     <row r="108">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
-      <c r="C108" s="1"/>
+      <c r="C108" s="1" t="str">
+        <v>王道商業銀行股份有限公司</v>
+      </c>
       <c r="D108" s="1"/>
       <c r="E108" s="1" t="str">
         <v>一碼付／UNIONPAY SecurePay</v>
@@ -17845,14 +18395,18 @@
       <c r="AG108" s="1"/>
       <c r="AH108" s="1"/>
       <c r="AI108" s="1"/>
-      <c r="AJ108" s="1"/>
+      <c r="AJ108" s="1" t="str">
+        <v>王道商業銀行股份有限公司</v>
+      </c>
       <c r="AK108" s="1"/>
       <c r="AL108" s="1"/>
     </row>
     <row r="109">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
-      <c r="C109" s="1"/>
+      <c r="C109" s="1" t="str">
+        <v>國家開發銀行</v>
+      </c>
       <c r="D109" s="1"/>
       <c r="E109" s="1" t="str">
         <v>一碼付／VISA Click To Pay</v>
@@ -17887,14 +18441,18 @@
       <c r="AG109" s="1"/>
       <c r="AH109" s="1"/>
       <c r="AI109" s="1"/>
-      <c r="AJ109" s="1"/>
+      <c r="AJ109" s="1" t="str">
+        <v>國家開發銀行</v>
+      </c>
       <c r="AK109" s="1"/>
       <c r="AL109" s="1"/>
     </row>
     <row r="110">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
-      <c r="C110" s="1"/>
+      <c r="C110" s="1" t="str">
+        <v>FIRST ABU DHABI BANK PJSC</v>
+      </c>
       <c r="D110" s="1"/>
       <c r="E110" s="1" t="str">
         <v>一碼付／MASTERCARD Click To Pay</v>
@@ -17929,14 +18487,18 @@
       <c r="AG110" s="1"/>
       <c r="AH110" s="1"/>
       <c r="AI110" s="1"/>
-      <c r="AJ110" s="1"/>
+      <c r="AJ110" s="1" t="str">
+        <v>FIRST ABU DHABI BANK PJSC</v>
+      </c>
       <c r="AK110" s="1"/>
       <c r="AL110" s="1"/>
     </row>
     <row r="111">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
-      <c r="C111" s="1"/>
+      <c r="C111" s="1" t="str">
+        <v>BANK J. SAFRA SARASIN LTD.</v>
+      </c>
       <c r="D111" s="1"/>
       <c r="E111" s="1" t="str">
         <v>一碼付／VISA Apple Pay</v>
@@ -17971,14 +18533,18 @@
       <c r="AG111" s="1"/>
       <c r="AH111" s="1"/>
       <c r="AI111" s="1"/>
-      <c r="AJ111" s="1"/>
+      <c r="AJ111" s="1" t="str">
+        <v>BANK J. SAFRA SARASIN LTD.</v>
+      </c>
       <c r="AK111" s="1"/>
       <c r="AL111" s="1"/>
     </row>
     <row r="112">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
-      <c r="C112" s="1"/>
+      <c r="C112" s="1" t="str">
+        <v>HDFC BANK LIMITED</v>
+      </c>
       <c r="D112" s="1"/>
       <c r="E112" s="1" t="str">
         <v>一碼付／MASTERCARD Apple Pay</v>
@@ -18013,14 +18579,18 @@
       <c r="AG112" s="1"/>
       <c r="AH112" s="1"/>
       <c r="AI112" s="1"/>
-      <c r="AJ112" s="1"/>
+      <c r="AJ112" s="1" t="str">
+        <v>HDFC BANK LIMITED</v>
+      </c>
       <c r="AK112" s="1"/>
       <c r="AL112" s="1"/>
     </row>
     <row r="113">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
-      <c r="C113" s="1"/>
+      <c r="C113" s="1" t="str">
+        <v>UNION BANCAIRE PRIVEE, UBP SA</v>
+      </c>
       <c r="D113" s="1"/>
       <c r="E113" s="1" t="str">
         <v>一碼付／VISA Google Pay</v>
@@ -18055,14 +18625,18 @@
       <c r="AG113" s="1"/>
       <c r="AH113" s="1"/>
       <c r="AI113" s="1"/>
-      <c r="AJ113" s="1"/>
+      <c r="AJ113" s="1" t="str">
+        <v>UNION BANCAIRE PRIVEE, UBP SA</v>
+      </c>
       <c r="AK113" s="1"/>
       <c r="AL113" s="1"/>
     </row>
     <row r="114">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
-      <c r="C114" s="1"/>
+      <c r="C114" s="1" t="str">
+        <v>SKANDINAVISKA ENSKILDA BANKEN AB</v>
+      </c>
       <c r="D114" s="1"/>
       <c r="E114" s="1" t="str">
         <v>一碼付／MASTERCARD Google Pay</v>
@@ -18097,14 +18671,18 @@
       <c r="AG114" s="1"/>
       <c r="AH114" s="1"/>
       <c r="AI114" s="1"/>
-      <c r="AJ114" s="1"/>
+      <c r="AJ114" s="1" t="str">
+        <v>SKANDINAVISKA ENSKILDA BANKEN AB</v>
+      </c>
       <c r="AK114" s="1"/>
       <c r="AL114" s="1"/>
     </row>
     <row r="115">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
-      <c r="C115" s="1"/>
+      <c r="C115" s="1" t="str">
+        <v>BANK JULIUS BAER &amp; CO. LTD.</v>
+      </c>
       <c r="D115" s="1"/>
       <c r="E115" s="1" t="str">
         <v>代扣／VISA 代扣</v>
@@ -18139,14 +18717,18 @@
       <c r="AG115" s="1"/>
       <c r="AH115" s="1"/>
       <c r="AI115" s="1"/>
-      <c r="AJ115" s="1"/>
+      <c r="AJ115" s="1" t="str">
+        <v>BANK JULIUS BAER &amp; CO. LTD.</v>
+      </c>
       <c r="AK115" s="1"/>
       <c r="AL115" s="1"/>
     </row>
     <row r="116">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
-      <c r="C116" s="1"/>
+      <c r="C116" s="1" t="str">
+        <v>法國工商銀行</v>
+      </c>
       <c r="D116" s="1"/>
       <c r="E116" s="1" t="str">
         <v>代扣／MASTERCARD 代扣</v>
@@ -18181,14 +18763,18 @@
       <c r="AG116" s="1"/>
       <c r="AH116" s="1"/>
       <c r="AI116" s="1"/>
-      <c r="AJ116" s="1"/>
+      <c r="AJ116" s="1" t="str">
+        <v>法國工商銀行</v>
+      </c>
       <c r="AK116" s="1"/>
       <c r="AL116" s="1"/>
     </row>
     <row r="117">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
-      <c r="C117" s="1"/>
+      <c r="C117" s="1" t="str">
+        <v>臺灣新光商業銀行股份有限公司</v>
+      </c>
       <c r="D117" s="1"/>
       <c r="E117" s="1" t="str">
         <v>代扣／微信代扣</v>
@@ -18223,14 +18809,18 @@
       <c r="AG117" s="1"/>
       <c r="AH117" s="1"/>
       <c r="AI117" s="1"/>
-      <c r="AJ117" s="1"/>
+      <c r="AJ117" s="1" t="str">
+        <v>臺灣新光商業銀行股份有限公司</v>
+      </c>
       <c r="AK117" s="1"/>
       <c r="AL117" s="1"/>
     </row>
     <row r="118">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
-      <c r="C118" s="1"/>
+      <c r="C118" s="1" t="str">
+        <v>中國銀行股份有限公司</v>
+      </c>
       <c r="D118" s="1"/>
       <c r="E118" s="1" t="str">
         <v>代扣／支付寶代扣</v>
@@ -18265,9 +18855,291 @@
       <c r="AG118" s="1"/>
       <c r="AH118" s="1"/>
       <c r="AI118" s="1"/>
-      <c r="AJ118" s="1"/>
+      <c r="AJ118" s="1" t="str">
+        <v>中國銀行股份有限公司</v>
+      </c>
       <c r="AK118" s="1"/>
       <c r="AL118" s="1"/>
+    </row>
+    <row r="119">
+      <c r="C119" t="str">
+        <v>CA INDOSUEZ (SWITZERLAND) SA</v>
+      </c>
+      <c r="AJ119" t="str">
+        <v>CA INDOSUEZ (SWITZERLAND) SA</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="C120" t="str">
+        <v>LGT皇家銀行(香港)</v>
+      </c>
+      <c r="AJ120" t="str">
+        <v>LGT皇家銀行(香港)</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="C121" t="str">
+        <v>上海浦東發展銀行股份有限公司</v>
+      </c>
+      <c r="AJ121" t="str">
+        <v>上海浦東發展銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="C122" t="str">
+        <v>中國民生銀行股份有限公司</v>
+      </c>
+      <c r="AJ122" t="str">
+        <v>中國民生銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="C123" t="str">
+        <v>廣發銀行股份有限公司</v>
+      </c>
+      <c r="AJ123" t="str">
+        <v>廣發銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="C124" t="str">
+        <v>渤海銀行股份有限公司</v>
+      </c>
+      <c r="AJ124" t="str">
+        <v>渤海銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="C125" t="str">
+        <v>BANQUE PICTET &amp; CIE SA</v>
+      </c>
+      <c r="AJ125" t="str">
+        <v>BANQUE PICTET &amp; CIE SA</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="C126" t="str">
+        <v>東莞銀行股份有限公司</v>
+      </c>
+      <c r="AJ126" t="str">
+        <v>東莞銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="C127" t="str">
+        <v>中國光大銀行股份有限公司</v>
+      </c>
+      <c r="AJ127" t="str">
+        <v>中國光大銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="C128" t="str">
+        <v>SUMITOMO MITSUI TRUST BANK, LIMITED</v>
+      </c>
+      <c r="AJ128" t="str">
+        <v>SUMITOMO MITSUI TRUST BANK, LIMITED</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="C129" t="str">
+        <v>上海銀行(香港)有限公司</v>
+      </c>
+      <c r="AJ129" t="str">
+        <v>上海銀行(香港)有限公司</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="C130" t="str">
+        <v>CIMB BANK BERHAD</v>
+      </c>
+      <c r="AJ130" t="str">
+        <v>CIMB BANK BERHAD</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" t="str">
+        <v>NONGHYUP BANK</v>
+      </c>
+      <c r="AJ131" t="str">
+        <v>NONGHYUP BANK</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="C132" t="str">
+        <v>興業銀行股份有限公司</v>
+      </c>
+      <c r="AJ132" t="str">
+        <v>興業銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="C133" t="str">
+        <v>元大商業銀行股份有限公司</v>
+      </c>
+      <c r="AJ133" t="str">
+        <v>元大商業銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="C134" t="str">
+        <v>MASHREQ BANK - PUBLIC SHAREHOLDING COMPANY</v>
+      </c>
+      <c r="AJ134" t="str">
+        <v>MASHREQ BANK - PUBLIC SHAREHOLDING COMPANY</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="C135" t="str">
+        <v>KOOKMIN BANK</v>
+      </c>
+      <c r="AJ135" t="str">
+        <v>KOOKMIN BANK</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="C136" t="str">
+        <v>交通銀行(香港)有限公司</v>
+      </c>
+      <c r="AJ136" t="str">
+        <v>交通銀行(香港)有限公司</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="C137" t="str">
+        <v>浙商銀行股份有限公司</v>
+      </c>
+      <c r="AJ137" t="str">
+        <v>浙商銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="C138" t="str">
+        <v>摩根士丹利銀行亞洲有限公司</v>
+      </c>
+      <c r="AJ138" t="str">
+        <v>摩根士丹利銀行亞洲有限公司</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="C139" t="str">
+        <v>平安銀行股份有限公司</v>
+      </c>
+      <c r="AJ139" t="str">
+        <v>平安銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="C140" t="str">
+        <v>華夏銀行股份有限公司</v>
+      </c>
+      <c r="AJ140" t="str">
+        <v>華夏銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="C141" t="str">
+        <v>眾安銀行有限公司</v>
+      </c>
+      <c r="AJ141" t="str">
+        <v>眾安銀行有限公司</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="C142" t="str">
+        <v>理慧銀行有限公司</v>
+      </c>
+      <c r="AJ142" t="str">
+        <v>理慧銀行有限公司</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="C143" t="str">
+        <v>MOX BANK LIMITED</v>
+      </c>
+      <c r="AJ143" t="str">
+        <v>MOX BANK LIMITED</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="C144" t="str">
+        <v>匯立銀行有限公司</v>
+      </c>
+      <c r="AJ144" t="str">
+        <v>匯立銀行有限公司</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="C145" t="str">
+        <v>富融銀行有限公司</v>
+      </c>
+      <c r="AJ145" t="str">
+        <v>富融銀行有限公司</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="C146" t="str">
+        <v>PAO BANK LIMITED</v>
+      </c>
+      <c r="AJ146" t="str">
+        <v>PAO BANK LIMITED</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="C147" t="str">
+        <v>螞蟻銀行(香港)有限公司</v>
+      </c>
+      <c r="AJ147" t="str">
+        <v>螞蟻銀行(香港)有限公司</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="C148" t="str">
+        <v>卡塔爾國家銀行</v>
+      </c>
+      <c r="AJ148" t="str">
+        <v>卡塔爾國家銀行</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="C149" t="str">
+        <v>天星銀行有限公司</v>
+      </c>
+      <c r="AJ149" t="str">
+        <v>天星銀行有限公司</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="C150" t="str">
+        <v>THE KOREA DEVELOPMENT BANK</v>
+      </c>
+      <c r="AJ150" t="str">
+        <v>THE KOREA DEVELOPMENT BANK</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="C151" t="str">
+        <v>中信銀行股份有限公司</v>
+      </c>
+      <c r="AJ151" t="str">
+        <v>中信銀行股份有限公司</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="C152" t="str">
+        <v>HONG KONG SECURITIES CLEARING COMPANY LIMITED</v>
+      </c>
+      <c r="AJ152" t="str">
+        <v>HONG KONG SECURITIES CLEARING COMPANY LIMITED</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="C153" t="str">
+        <v>CONTINUOUS LINKED SETTLEMENT BANK INTERNATIONAL</v>
+      </c>
+      <c r="AJ153" t="str">
+        <v>CONTINUOUS LINKED SETTLEMENT BANK INTERNATIONAL</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>